<commit_message>
#17 eSpark and Client BOM Updated acc to design
</commit_message>
<xml_diff>
--- a/Design Files/Ethernet-Module-v2.0/BOM/Client_BOM_Ethernet-Module-v2.0.xlsx
+++ b/Design Files/Ethernet-Module-v2.0/BOM/Client_BOM_Ethernet-Module-v2.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\chrisbyrd-esp32iotproduct\Design Files\Ethernet-Module-v2.0\Ethernet-Module-v2.0\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\chrisbyrd-esp32iotproduct\Design Files\Ethernet-Module-v2.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="150">
   <si>
     <t>Component list</t>
   </si>
@@ -183,9 +183,6 @@
     <t>RES SMD 1K OHM 1% 1/10W 0603</t>
   </si>
   <si>
-    <t>RES SMD 10K OHM 5% 1/10W 0603</t>
-  </si>
-  <si>
     <t>RES SMD 0R, 1%, 0.1W, 0603</t>
   </si>
   <si>
@@ -282,9 +279,6 @@
     <t>RC0603FR-071KL</t>
   </si>
   <si>
-    <t>AC0603JR-0710KL</t>
-  </si>
-  <si>
     <t>RC0603FR-070RL</t>
   </si>
   <si>
@@ -330,139 +324,151 @@
     <t>Taiyo Yuden</t>
   </si>
   <si>
+    <t>TECH PUBLIC</t>
+  </si>
+  <si>
+    <t>ON Semiconductor / Fairchild</t>
+  </si>
+  <si>
+    <t>WIZNET</t>
+  </si>
+  <si>
+    <t>Littelfuse</t>
+  </si>
+  <si>
+    <t>NDK</t>
+  </si>
+  <si>
+    <t>22uF</t>
+  </si>
+  <si>
+    <t>0.1uF</t>
+  </si>
+  <si>
+    <t>10uF</t>
+  </si>
+  <si>
+    <t>6.8nF</t>
+  </si>
+  <si>
+    <t>22nF</t>
+  </si>
+  <si>
+    <t>10nF</t>
+  </si>
+  <si>
+    <t>4.7uF</t>
+  </si>
+  <si>
+    <t>12pF</t>
+  </si>
+  <si>
+    <t>1K</t>
+  </si>
+  <si>
+    <t>10K</t>
+  </si>
+  <si>
+    <t>0R</t>
+  </si>
+  <si>
+    <t>49.9R</t>
+  </si>
+  <si>
+    <t>10R</t>
+  </si>
+  <si>
+    <t>33R</t>
+  </si>
+  <si>
+    <t>330R</t>
+  </si>
+  <si>
+    <t>1M</t>
+  </si>
+  <si>
+    <t>12.4K</t>
+  </si>
+  <si>
+    <t>25MHZ</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Alternate Part Number</t>
+  </si>
+  <si>
+    <t>Quantity (5 Boards)</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>DO NOT MOUNT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mini PCIe SMD Pad </t>
+  </si>
+  <si>
+    <t>Unit Cost (5 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (5 Boards)</t>
+  </si>
+  <si>
+    <t>Links</t>
+  </si>
+  <si>
+    <t>Digikey</t>
+  </si>
+  <si>
+    <t>Custom Supplier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Component Cost </t>
+  </si>
+  <si>
+    <t>Single Board Cost</t>
+  </si>
+  <si>
+    <t>Bill of Materials for Project [Ethernet-Module-v2.0.]</t>
+  </si>
+  <si>
+    <t>Ethernet-Module-v2.0.</t>
+  </si>
+  <si>
+    <t>R2, R9, R12, R17, R18, R19, R22, R23, R24, R25, R26, R27, R29, R30, R31, R32</t>
+  </si>
+  <si>
+    <t>CONN JACK 1PORT 100 BASE-T PCB</t>
+  </si>
+  <si>
+    <t>ARJM11D7-114-AB-EW2</t>
+  </si>
+  <si>
     <t>Abracon</t>
   </si>
   <si>
-    <t>TECH PUBLIC</t>
-  </si>
-  <si>
-    <t>ON Semiconductor / Fairchild</t>
-  </si>
-  <si>
-    <t>WIZNET</t>
-  </si>
-  <si>
-    <t>Littelfuse</t>
-  </si>
-  <si>
-    <t>NDK</t>
-  </si>
-  <si>
-    <t>22uF</t>
-  </si>
-  <si>
-    <t>0.1uF</t>
-  </si>
-  <si>
-    <t>10uF</t>
-  </si>
-  <si>
-    <t>6.8nF</t>
-  </si>
-  <si>
-    <t>22nF</t>
-  </si>
-  <si>
-    <t>10nF</t>
-  </si>
-  <si>
-    <t>4.7uF</t>
-  </si>
-  <si>
-    <t>12pF</t>
-  </si>
-  <si>
-    <t>1K</t>
-  </si>
-  <si>
-    <t>10K</t>
-  </si>
-  <si>
-    <t>0R</t>
-  </si>
-  <si>
-    <t>49.9R</t>
-  </si>
-  <si>
-    <t>10R</t>
-  </si>
-  <si>
-    <t>33R</t>
-  </si>
-  <si>
-    <t>330R</t>
-  </si>
-  <si>
-    <t>1M</t>
-  </si>
-  <si>
-    <t>12.4K</t>
-  </si>
-  <si>
-    <t>25MHZ</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Alternate Part Number</t>
-  </si>
-  <si>
-    <t>Quantity (5 Boards)</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>Custom</t>
-  </si>
-  <si>
-    <t>DO NOT MOUNT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mini PCIe SMD Pad </t>
-  </si>
-  <si>
-    <t>Unit Cost (5 Boards)</t>
-  </si>
-  <si>
-    <t>Total Cost (5 Boards)</t>
-  </si>
-  <si>
-    <t>Links</t>
-  </si>
-  <si>
-    <t>Digikey</t>
-  </si>
-  <si>
-    <t>Custom Supplier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Component Cost </t>
-  </si>
-  <si>
-    <t>Single Board Cost</t>
-  </si>
-  <si>
-    <t>ARJM11D7-114-AB-EW2</t>
-  </si>
-  <si>
-    <t>CONN JACK 1PORT 100 BASE-T PCB</t>
-  </si>
-  <si>
-    <t>Bill of Materials for Project [Ethernet-Module-v2.0.]</t>
-  </si>
-  <si>
-    <t>Ethernet-Module-v2.0.</t>
-  </si>
-  <si>
-    <t>R2, R9, R12, R17, R18, R19, R22, R23, R24, R25, R26, R27, R29, R30, R31, R32</t>
+    <t>Mouser</t>
+  </si>
+  <si>
+    <t>RES SMD 10K OHM 1% 1/20W 0201</t>
+  </si>
+  <si>
+    <t>Res-0201</t>
+  </si>
+  <si>
+    <t>RC0201FR-0710KL</t>
   </si>
 </sst>
 </file>
@@ -890,7 +896,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1085,6 +1091,15 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1474,7 +1489,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -1496,7 +1511,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -1518,7 +1533,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1622,37 +1637,37 @@
         <v>40</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="J9" s="29" t="s">
+        <v>125</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>124</v>
+      </c>
+      <c r="L9" s="29" t="s">
         <v>128</v>
       </c>
-      <c r="K9" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="L9" s="29" t="s">
-        <v>131</v>
-      </c>
       <c r="M9" s="29" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="N9" s="29" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="O9" s="29" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="P9" s="29" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1671,19 +1686,19 @@
         <v>41</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J10" s="36" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="K10" s="36">
         <v>2</v>
@@ -1693,7 +1708,7 @@
         <v>10</v>
       </c>
       <c r="M10" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N10" s="62">
         <v>0.68</v>
@@ -1720,19 +1735,19 @@
         <v>42</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G11" s="39" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J11" s="38" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="K11" s="38">
         <v>7</v>
@@ -1742,7 +1757,7 @@
         <v>35</v>
       </c>
       <c r="M11" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N11" s="63">
         <v>0.1</v>
@@ -1769,19 +1784,19 @@
         <v>43</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="J12" s="36" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="K12" s="36">
         <v>2</v>
@@ -1791,7 +1806,7 @@
         <v>10</v>
       </c>
       <c r="M12" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N12" s="62">
         <v>0.75</v>
@@ -1818,19 +1833,19 @@
         <v>44</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G13" s="39" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H13" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="J13" s="38" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="K13" s="38">
         <v>2</v>
@@ -1840,7 +1855,7 @@
         <v>10</v>
       </c>
       <c r="M13" s="61" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="N13" s="63"/>
       <c r="O13" s="62">
@@ -1865,19 +1880,19 @@
         <v>45</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G14" s="37" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="J14" s="36" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="K14" s="36">
         <v>1</v>
@@ -1887,7 +1902,7 @@
         <v>5</v>
       </c>
       <c r="M14" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N14" s="62">
         <v>0.1</v>
@@ -1914,19 +1929,19 @@
         <v>46</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G15" s="39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H15" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J15" s="38" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="K15" s="38">
         <v>2</v>
@@ -1936,7 +1951,7 @@
         <v>10</v>
       </c>
       <c r="M15" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N15" s="63">
         <v>9.7000000000000003E-2</v>
@@ -1963,19 +1978,19 @@
         <v>47</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="J16" s="36" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="K16" s="36">
         <v>1</v>
@@ -1985,7 +2000,7 @@
         <v>5</v>
       </c>
       <c r="M16" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N16" s="62">
         <v>0.32</v>
@@ -2012,19 +2027,19 @@
         <v>48</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G17" s="39" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H17" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="J17" s="38" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="K17" s="38">
         <v>2</v>
@@ -2034,7 +2049,7 @@
         <v>10</v>
       </c>
       <c r="M17" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N17" s="63">
         <v>0.11</v>
@@ -2061,19 +2076,19 @@
         <v>49</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G18" s="37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H18" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J18" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K18" s="36">
         <v>2</v>
@@ -2083,7 +2098,7 @@
         <v>10</v>
       </c>
       <c r="M18" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N18" s="62">
         <v>0.38</v>
@@ -2103,26 +2118,26 @@
       <c r="C19" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="D19" s="38" t="s">
+      <c r="D19" s="72" t="s">
         <v>25</v>
       </c>
-      <c r="E19" s="39" t="s">
+      <c r="E19" s="72" t="s">
+        <v>143</v>
+      </c>
+      <c r="F19" s="72" t="s">
+        <v>130</v>
+      </c>
+      <c r="G19" s="72" t="s">
         <v>144</v>
       </c>
-      <c r="F19" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="G19" s="39" t="s">
-        <v>143</v>
-      </c>
       <c r="H19" s="36" t="s">
-        <v>129</v>
-      </c>
-      <c r="I19" s="38" t="s">
-        <v>103</v>
+        <v>126</v>
+      </c>
+      <c r="I19" s="72" t="s">
+        <v>145</v>
       </c>
       <c r="J19" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K19" s="38">
         <v>1</v>
@@ -2131,15 +2146,15 @@
         <f t="shared" ref="L19" si="6">K19*5</f>
         <v>5</v>
       </c>
-      <c r="M19" s="61" t="s">
-        <v>139</v>
-      </c>
-      <c r="N19" s="63">
-        <v>3.46</v>
+      <c r="M19" s="73" t="s">
+        <v>146</v>
+      </c>
+      <c r="N19" s="74">
+        <v>3.47</v>
       </c>
       <c r="O19" s="62">
         <f t="shared" si="2"/>
-        <v>17.3</v>
+        <v>17.350000000000001</v>
       </c>
       <c r="P19" s="38"/>
     </row>
@@ -2150,7 +2165,7 @@
         <v>11</v>
       </c>
       <c r="C20" s="57" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D20" s="55" t="s">
         <v>26</v>
@@ -2159,19 +2174,19 @@
         <v>50</v>
       </c>
       <c r="F20" s="55" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="G20" s="59" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="H20" s="55" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I20" s="55" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="J20" s="55" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K20" s="55">
         <v>1</v>
@@ -2181,14 +2196,14 @@
         <v>5</v>
       </c>
       <c r="M20" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="N20" s="64"/>
       <c r="O20" s="62" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="P20" s="56" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="21" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2207,19 +2222,19 @@
         <v>51</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G21" s="39" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="J21" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K21" s="38">
         <v>1</v>
@@ -2229,7 +2244,7 @@
         <v>5</v>
       </c>
       <c r="M21" s="61" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="N21" s="63"/>
       <c r="O21" s="62">
@@ -2254,19 +2269,19 @@
         <v>52</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G22" s="37" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H22" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I22" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="J22" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K22" s="36">
         <v>1</v>
@@ -2276,7 +2291,7 @@
         <v>5</v>
       </c>
       <c r="M22" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N22" s="62">
         <v>0.46</v>
@@ -2303,19 +2318,19 @@
         <v>53</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G23" s="39" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I23" s="38" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J23" s="38" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="K23" s="38">
         <v>1</v>
@@ -2325,7 +2340,7 @@
         <v>5</v>
       </c>
       <c r="M23" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N23" s="63">
         <v>0.1</v>
@@ -2346,25 +2361,25 @@
         <v>11</v>
       </c>
       <c r="D24" s="36" t="s">
+        <v>142</v>
+      </c>
+      <c r="E24" s="36" t="s">
         <v>147</v>
       </c>
-      <c r="E24" s="37" t="s">
-        <v>54</v>
-      </c>
       <c r="F24" s="36" t="s">
-        <v>70</v>
-      </c>
-      <c r="G24" s="37" t="s">
-        <v>87</v>
+        <v>148</v>
+      </c>
+      <c r="G24" s="36" t="s">
+        <v>149</v>
       </c>
       <c r="H24" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I24" s="36" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J24" s="36" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="K24" s="36">
         <v>16</v>
@@ -2374,7 +2389,7 @@
         <v>80</v>
       </c>
       <c r="M24" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N24" s="63">
         <v>0.1</v>
@@ -2398,22 +2413,22 @@
         <v>30</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F25" s="38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G25" s="39" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H25" s="38" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I25" s="38" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J25" s="38" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="K25" s="38">
         <v>2</v>
@@ -2423,7 +2438,7 @@
         <v>10</v>
       </c>
       <c r="M25" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N25" s="63">
         <v>0.1</v>
@@ -2447,22 +2462,22 @@
         <v>31</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G26" s="37" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H26" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I26" s="36" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J26" s="36" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="K26" s="36">
         <v>4</v>
@@ -2472,7 +2487,7 @@
         <v>20</v>
       </c>
       <c r="M26" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N26" s="63">
         <v>0.1</v>
@@ -2496,22 +2511,22 @@
         <v>32</v>
       </c>
       <c r="E27" s="39" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F27" s="38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G27" s="39" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="H27" s="38" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I27" s="38" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J27" s="38" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="K27" s="38">
         <v>1</v>
@@ -2521,7 +2536,7 @@
         <v>5</v>
       </c>
       <c r="M27" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N27" s="63">
         <v>0.1</v>
@@ -2545,22 +2560,22 @@
         <v>33</v>
       </c>
       <c r="E28" s="37" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G28" s="37" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H28" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I28" s="36" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J28" s="36" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="K28" s="36">
         <v>4</v>
@@ -2570,7 +2585,7 @@
         <v>20</v>
       </c>
       <c r="M28" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N28" s="63">
         <v>0.1</v>
@@ -2594,22 +2609,22 @@
         <v>34</v>
       </c>
       <c r="E29" s="39" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G29" s="39" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H29" s="38" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I29" s="38" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J29" s="38" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="K29" s="38">
         <v>2</v>
@@ -2619,7 +2634,7 @@
         <v>10</v>
       </c>
       <c r="M29" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N29" s="63">
         <v>0.1</v>
@@ -2643,22 +2658,22 @@
         <v>35</v>
       </c>
       <c r="E30" s="37" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G30" s="37" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H30" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I30" s="36" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J30" s="36" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="K30" s="36">
         <v>1</v>
@@ -2668,7 +2683,7 @@
         <v>5</v>
       </c>
       <c r="M30" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N30" s="63">
         <v>0.1</v>
@@ -2692,22 +2707,22 @@
         <v>36</v>
       </c>
       <c r="E31" s="39" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F31" s="38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G31" s="39" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="H31" s="38" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I31" s="38" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J31" s="38" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="K31" s="38">
         <v>1</v>
@@ -2717,7 +2732,7 @@
         <v>5</v>
       </c>
       <c r="M31" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N31" s="63">
         <v>0.1</v>
@@ -2741,22 +2756,22 @@
         <v>37</v>
       </c>
       <c r="E32" s="37" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G32" s="37" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H32" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I32" s="36" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="J32" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K32" s="36">
         <v>1</v>
@@ -2766,7 +2781,7 @@
         <v>5</v>
       </c>
       <c r="M32" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N32" s="62">
         <v>3.85</v>
@@ -2790,22 +2805,22 @@
         <v>38</v>
       </c>
       <c r="E33" s="39" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F33" s="38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G33" s="39" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="H33" s="38" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I33" s="38" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="J33" s="38" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K33" s="38">
         <v>1</v>
@@ -2815,7 +2830,7 @@
         <v>5</v>
       </c>
       <c r="M33" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N33" s="63">
         <v>0.87</v>
@@ -2839,22 +2854,22 @@
         <v>39</v>
       </c>
       <c r="E34" s="37" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="G34" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H34" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I34" s="36" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="J34" s="36" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="K34" s="36">
         <v>1</v>
@@ -2864,7 +2879,7 @@
         <v>5</v>
       </c>
       <c r="M34" s="61" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N34" s="62">
         <v>0.59</v>
@@ -2888,13 +2903,13 @@
       <c r="J35" s="35"/>
       <c r="K35" s="35"/>
       <c r="L35" s="70" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="M35" s="71"/>
       <c r="N35" s="71"/>
       <c r="O35" s="65">
         <f>SUM(O10:O34)</f>
-        <v>87.92</v>
+        <v>87.97</v>
       </c>
       <c r="P35" s="41"/>
     </row>
@@ -2911,13 +2926,13 @@
       <c r="J36" s="9"/>
       <c r="K36" s="9"/>
       <c r="L36" s="70" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="M36" s="71"/>
       <c r="N36" s="71"/>
       <c r="O36" s="66">
         <f>O35/5</f>
-        <v>17.584</v>
+        <v>17.594000000000001</v>
       </c>
       <c r="P36" s="42"/>
     </row>
@@ -2939,18 +2954,18 @@
     <hyperlink ref="M18" r:id="rId8"/>
     <hyperlink ref="M22" r:id="rId9"/>
     <hyperlink ref="M23" r:id="rId10"/>
-    <hyperlink ref="M24" r:id="rId11"/>
-    <hyperlink ref="M25" r:id="rId12"/>
-    <hyperlink ref="M26" r:id="rId13"/>
-    <hyperlink ref="M27" r:id="rId14"/>
-    <hyperlink ref="M28" r:id="rId15"/>
-    <hyperlink ref="M29" r:id="rId16"/>
-    <hyperlink ref="M30" r:id="rId17"/>
-    <hyperlink ref="M31" r:id="rId18"/>
-    <hyperlink ref="M32" r:id="rId19"/>
-    <hyperlink ref="M33" r:id="rId20"/>
-    <hyperlink ref="M34" r:id="rId21"/>
-    <hyperlink ref="M19" r:id="rId22"/>
+    <hyperlink ref="M25" r:id="rId11"/>
+    <hyperlink ref="M26" r:id="rId12"/>
+    <hyperlink ref="M27" r:id="rId13"/>
+    <hyperlink ref="M28" r:id="rId14"/>
+    <hyperlink ref="M29" r:id="rId15"/>
+    <hyperlink ref="M30" r:id="rId16"/>
+    <hyperlink ref="M31" r:id="rId17"/>
+    <hyperlink ref="M32" r:id="rId18"/>
+    <hyperlink ref="M33" r:id="rId19"/>
+    <hyperlink ref="M34" r:id="rId20"/>
+    <hyperlink ref="M19" r:id="rId21"/>
+    <hyperlink ref="M24" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId23"/>

</xml_diff>

<commit_message>
#17 0R resistor added 10k resistor deleted.
</commit_message>
<xml_diff>
--- a/Design Files/Ethernet-Module-v2.0/BOM/Client_BOM_Ethernet-Module-v2.0.xlsx
+++ b/Design Files/Ethernet-Module-v2.0/BOM/Client_BOM_Ethernet-Module-v2.0.xlsx
@@ -111,9 +111,6 @@
     <t>R1</t>
   </si>
   <si>
-    <t>R3, R21</t>
-  </si>
-  <si>
     <t>R4, R5, R15, R16</t>
   </si>
   <si>
@@ -447,9 +444,6 @@
     <t>Ethernet-Module-v2.0.</t>
   </si>
   <si>
-    <t>R2, R9, R12, R17, R18, R19, R22, R23, R24, R25, R26, R27, R29, R30, R31, R32</t>
-  </si>
-  <si>
     <t>CONN JACK 1PORT 100 BASE-T PCB</t>
   </si>
   <si>
@@ -469,6 +463,12 @@
   </si>
   <si>
     <t>RC0201FR-0710KL</t>
+  </si>
+  <si>
+    <t>R2, R9, R12, R17, R18, R19, R22, R23, R24, R25, R26, R27</t>
+  </si>
+  <si>
+    <t>R3, R21, R29</t>
   </si>
 </sst>
 </file>
@@ -1075,6 +1075,15 @@
     <xf numFmtId="166" fontId="14" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1091,15 +1100,6 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1472,13 +1472,13 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
+      <c r="N1" s="70"/>
+      <c r="O1" s="70"/>
+      <c r="P1" s="70"/>
     </row>
     <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -1522,7 +1522,7 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="68"/>
+      <c r="P3" s="71"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1544,7 +1544,7 @@
       <c r="M4" s="60"/>
       <c r="N4" s="60"/>
       <c r="O4" s="60"/>
-      <c r="P4" s="69"/>
+      <c r="P4" s="72"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1566,7 +1566,7 @@
       <c r="M5" s="60"/>
       <c r="N5" s="60"/>
       <c r="O5" s="60"/>
-      <c r="P5" s="69"/>
+      <c r="P5" s="72"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1584,7 +1584,7 @@
       <c r="M6" s="60"/>
       <c r="N6" s="60"/>
       <c r="O6" s="60"/>
-      <c r="P6" s="69"/>
+      <c r="P6" s="72"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1602,7 +1602,7 @@
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
-      <c r="P7" s="69"/>
+      <c r="P7" s="72"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1620,7 +1620,7 @@
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
-      <c r="P8" s="69"/>
+      <c r="P8" s="72"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1634,40 +1634,40 @@
         <v>15</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H9" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="I9" s="29" t="s">
+        <v>94</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>124</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="L9" s="29" t="s">
         <v>127</v>
       </c>
-      <c r="I9" s="29" t="s">
-        <v>95</v>
-      </c>
-      <c r="J9" s="29" t="s">
-        <v>125</v>
-      </c>
-      <c r="K9" s="29" t="s">
-        <v>124</v>
-      </c>
-      <c r="L9" s="29" t="s">
+      <c r="M9" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="N9" s="29" t="s">
+        <v>132</v>
+      </c>
+      <c r="O9" s="29" t="s">
+        <v>133</v>
+      </c>
+      <c r="P9" s="29" t="s">
         <v>128</v>
-      </c>
-      <c r="M9" s="29" t="s">
-        <v>135</v>
-      </c>
-      <c r="N9" s="29" t="s">
-        <v>133</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="P9" s="29" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1683,22 +1683,22 @@
         <v>16</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J10" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K10" s="36">
         <v>2</v>
@@ -1708,7 +1708,7 @@
         <v>10</v>
       </c>
       <c r="M10" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N10" s="62">
         <v>0.68</v>
@@ -1732,22 +1732,22 @@
         <v>17</v>
       </c>
       <c r="E11" s="39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G11" s="39" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J11" s="38" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="K11" s="38">
         <v>7</v>
@@ -1757,7 +1757,7 @@
         <v>35</v>
       </c>
       <c r="M11" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N11" s="63">
         <v>0.1</v>
@@ -1781,22 +1781,22 @@
         <v>18</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J12" s="36" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K12" s="36">
         <v>2</v>
@@ -1806,7 +1806,7 @@
         <v>10</v>
       </c>
       <c r="M12" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N12" s="62">
         <v>0.75</v>
@@ -1830,22 +1830,22 @@
         <v>19</v>
       </c>
       <c r="E13" s="39" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G13" s="39" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H13" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J13" s="38" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K13" s="38">
         <v>2</v>
@@ -1855,7 +1855,7 @@
         <v>10</v>
       </c>
       <c r="M13" s="61" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="N13" s="63"/>
       <c r="O13" s="62">
@@ -1877,22 +1877,22 @@
         <v>20</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G14" s="37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J14" s="36" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K14" s="36">
         <v>1</v>
@@ -1902,7 +1902,7 @@
         <v>5</v>
       </c>
       <c r="M14" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N14" s="62">
         <v>0.1</v>
@@ -1926,22 +1926,22 @@
         <v>21</v>
       </c>
       <c r="E15" s="39" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G15" s="39" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H15" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J15" s="38" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K15" s="38">
         <v>2</v>
@@ -1951,7 +1951,7 @@
         <v>10</v>
       </c>
       <c r="M15" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N15" s="63">
         <v>9.7000000000000003E-2</v>
@@ -1975,22 +1975,22 @@
         <v>22</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J16" s="36" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K16" s="36">
         <v>1</v>
@@ -2000,7 +2000,7 @@
         <v>5</v>
       </c>
       <c r="M16" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N16" s="62">
         <v>0.32</v>
@@ -2024,22 +2024,22 @@
         <v>23</v>
       </c>
       <c r="E17" s="39" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G17" s="39" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H17" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J17" s="38" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="K17" s="38">
         <v>2</v>
@@ -2049,7 +2049,7 @@
         <v>10</v>
       </c>
       <c r="M17" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N17" s="63">
         <v>0.11</v>
@@ -2073,22 +2073,22 @@
         <v>24</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G18" s="37" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H18" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J18" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K18" s="36">
         <v>2</v>
@@ -2098,7 +2098,7 @@
         <v>10</v>
       </c>
       <c r="M18" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N18" s="62">
         <v>0.38</v>
@@ -2118,26 +2118,26 @@
       <c r="C19" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="D19" s="72" t="s">
+      <c r="D19" s="67" t="s">
         <v>25</v>
       </c>
-      <c r="E19" s="72" t="s">
+      <c r="E19" s="67" t="s">
+        <v>141</v>
+      </c>
+      <c r="F19" s="67" t="s">
+        <v>129</v>
+      </c>
+      <c r="G19" s="67" t="s">
+        <v>142</v>
+      </c>
+      <c r="H19" s="36" t="s">
+        <v>125</v>
+      </c>
+      <c r="I19" s="67" t="s">
         <v>143</v>
       </c>
-      <c r="F19" s="72" t="s">
-        <v>130</v>
-      </c>
-      <c r="G19" s="72" t="s">
-        <v>144</v>
-      </c>
-      <c r="H19" s="36" t="s">
-        <v>126</v>
-      </c>
-      <c r="I19" s="72" t="s">
-        <v>145</v>
-      </c>
       <c r="J19" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K19" s="38">
         <v>1</v>
@@ -2146,10 +2146,10 @@
         <f t="shared" ref="L19" si="6">K19*5</f>
         <v>5</v>
       </c>
-      <c r="M19" s="73" t="s">
-        <v>146</v>
-      </c>
-      <c r="N19" s="74">
+      <c r="M19" s="68" t="s">
+        <v>144</v>
+      </c>
+      <c r="N19" s="69">
         <v>3.47</v>
       </c>
       <c r="O19" s="62">
@@ -2165,28 +2165,28 @@
         <v>11</v>
       </c>
       <c r="C20" s="57" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D20" s="55" t="s">
         <v>26</v>
       </c>
       <c r="E20" s="59" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F20" s="55" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G20" s="59" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H20" s="55" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I20" s="55" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J20" s="55" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K20" s="55">
         <v>1</v>
@@ -2196,14 +2196,14 @@
         <v>5</v>
       </c>
       <c r="M20" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="N20" s="64"/>
       <c r="O20" s="62" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P20" s="56" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="21" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2219,22 +2219,22 @@
         <v>27</v>
       </c>
       <c r="E21" s="39" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G21" s="39" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J21" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K21" s="38">
         <v>1</v>
@@ -2244,7 +2244,7 @@
         <v>5</v>
       </c>
       <c r="M21" s="61" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="N21" s="63"/>
       <c r="O21" s="62">
@@ -2266,22 +2266,22 @@
         <v>28</v>
       </c>
       <c r="E22" s="37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G22" s="37" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H22" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I22" s="36" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J22" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K22" s="36">
         <v>1</v>
@@ -2291,7 +2291,7 @@
         <v>5</v>
       </c>
       <c r="M22" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N22" s="62">
         <v>0.46</v>
@@ -2315,22 +2315,22 @@
         <v>29</v>
       </c>
       <c r="E23" s="39" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G23" s="39" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I23" s="38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J23" s="38" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K23" s="38">
         <v>1</v>
@@ -2340,7 +2340,7 @@
         <v>5</v>
       </c>
       <c r="M23" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N23" s="63">
         <v>0.1</v>
@@ -2361,42 +2361,42 @@
         <v>11</v>
       </c>
       <c r="D24" s="36" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="E24" s="36" t="s">
+        <v>145</v>
+      </c>
+      <c r="F24" s="36" t="s">
+        <v>146</v>
+      </c>
+      <c r="G24" s="36" t="s">
         <v>147</v>
       </c>
-      <c r="F24" s="36" t="s">
-        <v>148</v>
-      </c>
-      <c r="G24" s="36" t="s">
-        <v>149</v>
-      </c>
       <c r="H24" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I24" s="36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J24" s="36" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K24" s="36">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="L24" s="37">
         <f>K24*5</f>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="M24" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N24" s="63">
         <v>0.1</v>
       </c>
       <c r="O24" s="62">
         <f t="shared" si="2"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P24" s="36"/>
     </row>
@@ -2410,42 +2410,42 @@
         <v>11</v>
       </c>
       <c r="D25" s="38" t="s">
-        <v>30</v>
+        <v>149</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F25" s="38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G25" s="39" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H25" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I25" s="38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J25" s="38" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K25" s="38">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L25" s="39">
         <f t="shared" ref="L25" si="9">K25*5</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="M25" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N25" s="63">
         <v>0.1</v>
       </c>
       <c r="O25" s="62">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="P25" s="38"/>
     </row>
@@ -2459,25 +2459,25 @@
         <v>11</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G26" s="37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H26" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I26" s="36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J26" s="36" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K26" s="36">
         <v>4</v>
@@ -2487,7 +2487,7 @@
         <v>20</v>
       </c>
       <c r="M26" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N26" s="63">
         <v>0.1</v>
@@ -2508,25 +2508,25 @@
         <v>11</v>
       </c>
       <c r="D27" s="38" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E27" s="39" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F27" s="38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G27" s="39" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H27" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I27" s="38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J27" s="38" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K27" s="38">
         <v>1</v>
@@ -2536,7 +2536,7 @@
         <v>5</v>
       </c>
       <c r="M27" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N27" s="63">
         <v>0.1</v>
@@ -2557,25 +2557,25 @@
         <v>11</v>
       </c>
       <c r="D28" s="36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E28" s="37" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G28" s="37" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H28" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I28" s="36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J28" s="36" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K28" s="36">
         <v>4</v>
@@ -2585,7 +2585,7 @@
         <v>20</v>
       </c>
       <c r="M28" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N28" s="63">
         <v>0.1</v>
@@ -2606,25 +2606,25 @@
         <v>11</v>
       </c>
       <c r="D29" s="38" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E29" s="39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G29" s="39" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H29" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I29" s="38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J29" s="38" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K29" s="38">
         <v>2</v>
@@ -2634,7 +2634,7 @@
         <v>10</v>
       </c>
       <c r="M29" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N29" s="63">
         <v>0.1</v>
@@ -2655,25 +2655,25 @@
         <v>11</v>
       </c>
       <c r="D30" s="36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E30" s="37" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G30" s="37" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H30" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I30" s="36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J30" s="36" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="K30" s="36">
         <v>1</v>
@@ -2683,7 +2683,7 @@
         <v>5</v>
       </c>
       <c r="M30" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N30" s="63">
         <v>0.1</v>
@@ -2704,25 +2704,25 @@
         <v>11</v>
       </c>
       <c r="D31" s="38" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E31" s="39" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F31" s="38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G31" s="39" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H31" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I31" s="38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J31" s="38" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K31" s="38">
         <v>1</v>
@@ -2732,7 +2732,7 @@
         <v>5</v>
       </c>
       <c r="M31" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N31" s="63">
         <v>0.1</v>
@@ -2753,25 +2753,25 @@
         <v>12</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E32" s="37" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G32" s="37" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H32" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I32" s="36" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J32" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K32" s="36">
         <v>1</v>
@@ -2781,7 +2781,7 @@
         <v>5</v>
       </c>
       <c r="M32" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N32" s="62">
         <v>3.85</v>
@@ -2802,25 +2802,25 @@
         <v>13</v>
       </c>
       <c r="D33" s="38" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E33" s="39" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F33" s="38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G33" s="39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H33" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I33" s="38" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J33" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K33" s="38">
         <v>1</v>
@@ -2830,7 +2830,7 @@
         <v>5</v>
       </c>
       <c r="M33" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N33" s="63">
         <v>0.87</v>
@@ -2851,25 +2851,25 @@
         <v>14</v>
       </c>
       <c r="D34" s="36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E34" s="37" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G34" s="37" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H34" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I34" s="36" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J34" s="36" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K34" s="36">
         <v>1</v>
@@ -2879,7 +2879,7 @@
         <v>5</v>
       </c>
       <c r="M34" s="61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N34" s="62">
         <v>0.59</v>
@@ -2902,14 +2902,14 @@
       <c r="I35" s="34"/>
       <c r="J35" s="35"/>
       <c r="K35" s="35"/>
-      <c r="L35" s="70" t="s">
-        <v>138</v>
-      </c>
-      <c r="M35" s="71"/>
-      <c r="N35" s="71"/>
+      <c r="L35" s="73" t="s">
+        <v>137</v>
+      </c>
+      <c r="M35" s="74"/>
+      <c r="N35" s="74"/>
       <c r="O35" s="65">
         <f>SUM(O10:O34)</f>
-        <v>87.97</v>
+        <v>86.47</v>
       </c>
       <c r="P35" s="41"/>
     </row>
@@ -2925,14 +2925,14 @@
       <c r="I36" s="9"/>
       <c r="J36" s="9"/>
       <c r="K36" s="9"/>
-      <c r="L36" s="70" t="s">
-        <v>139</v>
-      </c>
-      <c r="M36" s="71"/>
-      <c r="N36" s="71"/>
+      <c r="L36" s="73" t="s">
+        <v>138</v>
+      </c>
+      <c r="M36" s="74"/>
+      <c r="N36" s="74"/>
       <c r="O36" s="66">
         <f>O35/5</f>
-        <v>17.594000000000001</v>
+        <v>17.294</v>
       </c>
       <c r="P36" s="42"/>
     </row>

</xml_diff>

<commit_message>
#17 4.7K Resistor Added (R30) in BOM
</commit_message>
<xml_diff>
--- a/Design Files/Ethernet-Module-v2.0/BOM/Client_BOM_Ethernet-Module-v2.0.xlsx
+++ b/Design Files/Ethernet-Module-v2.0/BOM/Client_BOM_Ethernet-Module-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="155">
   <si>
     <t>Component list</t>
   </si>
@@ -469,6 +469,21 @@
   </si>
   <si>
     <t>R3, R21, R29</t>
+  </si>
+  <si>
+    <t>R30</t>
+  </si>
+  <si>
+    <t>RES 4.7K OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>Res-0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-074K7L</t>
+  </si>
+  <si>
+    <t>4.7K</t>
   </si>
 </sst>
 </file>
@@ -1443,7 +1458,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1722,7 +1737,7 @@
     <row r="11" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="50">
-        <f t="shared" ref="B11:B33" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B34" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="58" t="s">
@@ -1763,7 +1778,7 @@
         <v>0.1</v>
       </c>
       <c r="O11" s="62">
-        <f t="shared" ref="O11:O34" si="2">N11*L11</f>
+        <f t="shared" ref="O11:O35" si="2">N11*L11</f>
         <v>3.5</v>
       </c>
       <c r="P11" s="38"/>
@@ -2728,7 +2743,7 @@
         <v>1</v>
       </c>
       <c r="L31" s="39">
-        <f t="shared" ref="L31" si="12">K31*5</f>
+        <f t="shared" ref="L31:L32" si="12">K31*5</f>
         <v>5</v>
       </c>
       <c r="M31" s="61" t="s">
@@ -2746,202 +2761,251 @@
     <row r="32" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="50">
-        <f>ROW(B32) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C32" s="57" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="E32" s="37" t="s">
-        <v>60</v>
+        <v>150</v>
+      </c>
+      <c r="E32" s="36" t="s">
+        <v>151</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="G32" s="37" t="s">
-        <v>92</v>
+        <v>152</v>
+      </c>
+      <c r="G32" s="36" t="s">
+        <v>153</v>
       </c>
       <c r="H32" s="36" t="s">
         <v>125</v>
       </c>
       <c r="I32" s="36" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="J32" s="36" t="s">
-        <v>125</v>
+        <v>154</v>
       </c>
       <c r="K32" s="36">
         <v>1</v>
       </c>
-      <c r="L32" s="37">
-        <f>K32*5</f>
+      <c r="L32" s="39">
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="M32" s="61" t="s">
         <v>135</v>
       </c>
       <c r="N32" s="62">
-        <v>3.85</v>
+        <v>0.1</v>
       </c>
       <c r="O32" s="62">
         <f t="shared" si="2"/>
-        <v>19.25</v>
+        <v>0.5</v>
       </c>
       <c r="P32" s="36"/>
     </row>
     <row r="33" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B33) - ROW($B$9)</f>
         <v>24</v>
       </c>
-      <c r="C33" s="58" t="s">
-        <v>13</v>
-      </c>
-      <c r="D33" s="38" t="s">
-        <v>37</v>
-      </c>
-      <c r="E33" s="39" t="s">
-        <v>61</v>
-      </c>
-      <c r="F33" s="38" t="s">
-        <v>70</v>
-      </c>
-      <c r="G33" s="39" t="s">
-        <v>93</v>
-      </c>
-      <c r="H33" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="I33" s="38" t="s">
-        <v>103</v>
-      </c>
-      <c r="J33" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="K33" s="38">
+      <c r="C33" s="57" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E33" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="F33" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="G33" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="H33" s="36" t="s">
+        <v>125</v>
+      </c>
+      <c r="I33" s="36" t="s">
+        <v>102</v>
+      </c>
+      <c r="J33" s="36" t="s">
+        <v>125</v>
+      </c>
+      <c r="K33" s="36">
         <v>1</v>
       </c>
-      <c r="L33" s="39">
-        <f t="shared" ref="L33" si="13">K33*5</f>
+      <c r="L33" s="37">
+        <f>K33*5</f>
         <v>5</v>
       </c>
       <c r="M33" s="61" t="s">
         <v>135</v>
       </c>
-      <c r="N33" s="63">
-        <v>0.87</v>
+      <c r="N33" s="62">
+        <v>3.85</v>
       </c>
       <c r="O33" s="62">
         <f t="shared" si="2"/>
-        <v>4.3499999999999996</v>
-      </c>
-      <c r="P33" s="38"/>
+        <v>19.25</v>
+      </c>
+      <c r="P33" s="36"/>
     </row>
     <row r="34" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="50">
-        <f>ROW(B34) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C34" s="57" t="s">
-        <v>14</v>
-      </c>
-      <c r="D34" s="36" t="s">
-        <v>38</v>
-      </c>
-      <c r="E34" s="37" t="s">
-        <v>62</v>
-      </c>
-      <c r="F34" s="36" t="s">
-        <v>129</v>
-      </c>
-      <c r="G34" s="37" t="s">
-        <v>71</v>
-      </c>
-      <c r="H34" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="I34" s="36" t="s">
-        <v>104</v>
-      </c>
-      <c r="J34" s="36" t="s">
-        <v>122</v>
-      </c>
-      <c r="K34" s="36">
+      <c r="C34" s="58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="38" t="s">
+        <v>37</v>
+      </c>
+      <c r="E34" s="39" t="s">
+        <v>61</v>
+      </c>
+      <c r="F34" s="38" t="s">
+        <v>70</v>
+      </c>
+      <c r="G34" s="39" t="s">
+        <v>93</v>
+      </c>
+      <c r="H34" s="38" t="s">
+        <v>125</v>
+      </c>
+      <c r="I34" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="J34" s="38" t="s">
+        <v>125</v>
+      </c>
+      <c r="K34" s="38">
         <v>1</v>
       </c>
-      <c r="L34" s="37">
-        <f>K34*5</f>
+      <c r="L34" s="39">
+        <f t="shared" ref="L34" si="13">K34*5</f>
         <v>5</v>
       </c>
       <c r="M34" s="61" t="s">
         <v>135</v>
       </c>
-      <c r="N34" s="62">
-        <v>0.59</v>
+      <c r="N34" s="63">
+        <v>0.87</v>
       </c>
       <c r="O34" s="62">
         <f t="shared" si="2"/>
+        <v>4.3499999999999996</v>
+      </c>
+      <c r="P34" s="38"/>
+    </row>
+    <row r="35" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="1"/>
+      <c r="B35" s="50">
+        <f>ROW(B35) - ROW($B$9)</f>
+        <v>26</v>
+      </c>
+      <c r="C35" s="57" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="E35" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="F35" s="36" t="s">
+        <v>129</v>
+      </c>
+      <c r="G35" s="37" t="s">
+        <v>71</v>
+      </c>
+      <c r="H35" s="36" t="s">
+        <v>125</v>
+      </c>
+      <c r="I35" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="J35" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="K35" s="36">
+        <v>1</v>
+      </c>
+      <c r="L35" s="37">
+        <f>K35*5</f>
+        <v>5</v>
+      </c>
+      <c r="M35" s="61" t="s">
+        <v>135</v>
+      </c>
+      <c r="N35" s="62">
+        <v>0.59</v>
+      </c>
+      <c r="O35" s="62">
+        <f t="shared" si="2"/>
         <v>2.9499999999999997</v>
       </c>
-      <c r="P34" s="36"/>
-    </row>
-    <row r="35" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="1"/>
-      <c r="B35" s="31"/>
-      <c r="C35" s="48"/>
-      <c r="D35" s="32"/>
-      <c r="E35" s="33"/>
-      <c r="F35" s="34"/>
-      <c r="G35" s="35"/>
-      <c r="H35" s="35"/>
-      <c r="I35" s="34"/>
-      <c r="J35" s="35"/>
-      <c r="K35" s="35"/>
-      <c r="L35" s="73" t="s">
-        <v>137</v>
-      </c>
-      <c r="M35" s="74"/>
-      <c r="N35" s="74"/>
-      <c r="O35" s="65">
-        <f>SUM(O10:O34)</f>
-        <v>86.47</v>
-      </c>
-      <c r="P35" s="41"/>
+      <c r="P35" s="36"/>
     </row>
     <row r="36" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
-      <c r="B36" s="24"/>
-      <c r="C36" s="49"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
-      <c r="H36" s="9"/>
-      <c r="I36" s="9"/>
-      <c r="J36" s="9"/>
-      <c r="K36" s="9"/>
+      <c r="B36" s="31"/>
+      <c r="C36" s="48"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="33"/>
+      <c r="F36" s="34"/>
+      <c r="G36" s="35"/>
+      <c r="H36" s="35"/>
+      <c r="I36" s="34"/>
+      <c r="J36" s="35"/>
+      <c r="K36" s="35"/>
       <c r="L36" s="73" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="M36" s="74"/>
       <c r="N36" s="74"/>
-      <c r="O36" s="66">
-        <f>O35/5</f>
-        <v>17.294</v>
-      </c>
-      <c r="P36" s="42"/>
+      <c r="O36" s="65">
+        <f>SUM(O10:O35)</f>
+        <v>86.97</v>
+      </c>
+      <c r="P36" s="41"/>
+    </row>
+    <row r="37" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="1"/>
+      <c r="B37" s="24"/>
+      <c r="C37" s="49"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
+      <c r="I37" s="9"/>
+      <c r="J37" s="9"/>
+      <c r="K37" s="9"/>
+      <c r="L37" s="73" t="s">
+        <v>138</v>
+      </c>
+      <c r="M37" s="74"/>
+      <c r="N37" s="74"/>
+      <c r="O37" s="66">
+        <f>O36/5</f>
+        <v>17.393999999999998</v>
+      </c>
+      <c r="P37" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="J1:P1"/>
     <mergeCell ref="P3:P8"/>
-    <mergeCell ref="L35:N35"/>
     <mergeCell ref="L36:N36"/>
+    <mergeCell ref="L37:N37"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="M10" r:id="rId1"/>
@@ -2961,14 +3025,15 @@
     <hyperlink ref="M29" r:id="rId15"/>
     <hyperlink ref="M30" r:id="rId16"/>
     <hyperlink ref="M31" r:id="rId17"/>
-    <hyperlink ref="M32" r:id="rId18"/>
-    <hyperlink ref="M33" r:id="rId19"/>
-    <hyperlink ref="M34" r:id="rId20"/>
+    <hyperlink ref="M33" r:id="rId18"/>
+    <hyperlink ref="M34" r:id="rId19"/>
+    <hyperlink ref="M35" r:id="rId20"/>
     <hyperlink ref="M19" r:id="rId21"/>
     <hyperlink ref="M24" r:id="rId22"/>
+    <hyperlink ref="M32" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId23"/>
-  <drawing r:id="rId24"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId24"/>
+  <drawing r:id="rId25"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#17 Client BOM Updated.
</commit_message>
<xml_diff>
--- a/Design Files/Ethernet-Module-v2.0/BOM/Client_BOM_Ethernet-Module-v2.0.xlsx
+++ b/Design Files/Ethernet-Module-v2.0/BOM/Client_BOM_Ethernet-Module-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="158">
   <si>
     <t>Component list</t>
   </si>
@@ -132,9 +132,6 @@
     <t>U1</t>
   </si>
   <si>
-    <t>U2</t>
-  </si>
-  <si>
     <t>X1</t>
   </si>
   <si>
@@ -204,9 +201,6 @@
     <t>SPI LQFP-48(7x7) Ethernet ICs ROHS</t>
   </si>
   <si>
-    <t>TVS DIODE 5.5VWM 8.5VC SOT23-5</t>
-  </si>
-  <si>
     <t>SMD3225-4P Crystals ROHS</t>
   </si>
   <si>
@@ -231,9 +225,6 @@
     <t>48-LQFP (7x7)_</t>
   </si>
   <si>
-    <t>SOT-23-5</t>
-  </si>
-  <si>
     <t>NX3225GA-25MHZ-STD-CRG-2</t>
   </si>
   <si>
@@ -300,9 +291,6 @@
     <t>W5500</t>
   </si>
   <si>
-    <t>SP0504BAHTG</t>
-  </si>
-  <si>
     <t>Manufacturer</t>
   </si>
   <si>
@@ -496,6 +484,15 @@
   </si>
   <si>
     <t xml:space="preserve">Shengwei </t>
+  </si>
+  <si>
+    <t>D1, D2</t>
+  </si>
+  <si>
+    <t>TVS DIODE 5.5VWM 8.5VC SOT23-3</t>
+  </si>
+  <si>
+    <t>SP0502BAHTG</t>
   </si>
 </sst>
 </file>
@@ -1111,6 +1108,12 @@
     <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1127,12 +1130,6 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1505,13 +1502,13 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
-      <c r="P1" s="70"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="72"/>
+      <c r="L1" s="72"/>
+      <c r="M1" s="72"/>
+      <c r="N1" s="72"/>
+      <c r="O1" s="72"/>
+      <c r="P1" s="72"/>
     </row>
     <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1522,7 +1519,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -1544,7 +1541,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -1555,7 +1552,7 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="71"/>
+      <c r="P3" s="73"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1566,7 +1563,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1577,7 +1574,7 @@
       <c r="M4" s="60"/>
       <c r="N4" s="60"/>
       <c r="O4" s="60"/>
-      <c r="P4" s="72"/>
+      <c r="P4" s="74"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1599,7 +1596,7 @@
       <c r="M5" s="60"/>
       <c r="N5" s="60"/>
       <c r="O5" s="60"/>
-      <c r="P5" s="72"/>
+      <c r="P5" s="74"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1617,7 +1614,7 @@
       <c r="M6" s="60"/>
       <c r="N6" s="60"/>
       <c r="O6" s="60"/>
-      <c r="P6" s="72"/>
+      <c r="P6" s="74"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1635,7 +1632,7 @@
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
-      <c r="P7" s="72"/>
+      <c r="P7" s="74"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1653,7 +1650,7 @@
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
-      <c r="P8" s="72"/>
+      <c r="P8" s="74"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1667,40 +1664,40 @@
         <v>15</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="J9" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>119</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="M9" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="N9" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="O9" s="29" t="s">
+        <v>129</v>
+      </c>
+      <c r="P9" s="29" t="s">
         <v>124</v>
-      </c>
-      <c r="K9" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="L9" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="M9" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="N9" s="29" t="s">
-        <v>132</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>133</v>
-      </c>
-      <c r="P9" s="29" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1716,22 +1713,22 @@
         <v>16</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="J10" s="36" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="K10" s="36">
         <v>2</v>
@@ -1741,7 +1738,7 @@
         <v>10</v>
       </c>
       <c r="M10" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N10" s="62">
         <v>0.68</v>
@@ -1755,7 +1752,7 @@
     <row r="11" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="50">
-        <f t="shared" ref="B11:B34" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B33" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="58" t="s">
@@ -1765,22 +1762,22 @@
         <v>17</v>
       </c>
       <c r="E11" s="39" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G11" s="39" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="J11" s="38" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="K11" s="38">
         <v>7</v>
@@ -1790,7 +1787,7 @@
         <v>35</v>
       </c>
       <c r="M11" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N11" s="63">
         <v>0.1</v>
@@ -1814,22 +1811,22 @@
         <v>18</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="J12" s="36" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="K12" s="36">
         <v>2</v>
@@ -1839,7 +1836,7 @@
         <v>10</v>
       </c>
       <c r="M12" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N12" s="62">
         <v>0.75</v>
@@ -1863,22 +1860,22 @@
         <v>19</v>
       </c>
       <c r="E13" s="39" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G13" s="39" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="H13" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="J13" s="38" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="K13" s="38">
         <v>2</v>
@@ -1888,7 +1885,7 @@
         <v>10</v>
       </c>
       <c r="M13" s="61" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="N13" s="63"/>
       <c r="O13" s="62">
@@ -1910,22 +1907,22 @@
         <v>20</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G14" s="37" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="J14" s="36" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="K14" s="36">
         <v>1</v>
@@ -1935,7 +1932,7 @@
         <v>5</v>
       </c>
       <c r="M14" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N14" s="62">
         <v>0.1</v>
@@ -1959,22 +1956,22 @@
         <v>21</v>
       </c>
       <c r="E15" s="39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G15" s="39" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H15" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="J15" s="38" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="K15" s="38">
         <v>2</v>
@@ -1984,7 +1981,7 @@
         <v>10</v>
       </c>
       <c r="M15" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N15" s="63">
         <v>9.7000000000000003E-2</v>
@@ -2008,22 +2005,22 @@
         <v>22</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="J16" s="36" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="K16" s="36">
         <v>1</v>
@@ -2033,7 +2030,7 @@
         <v>5</v>
       </c>
       <c r="M16" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N16" s="62">
         <v>0.32</v>
@@ -2057,32 +2054,32 @@
         <v>23</v>
       </c>
       <c r="E17" s="39" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G17" s="39" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="H17" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="J17" s="38" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="K17" s="38">
         <v>2</v>
       </c>
       <c r="L17" s="39">
-        <f t="shared" ref="L17" si="5">K17*5</f>
+        <f t="shared" ref="L17:L18" si="5">K17*5</f>
         <v>10</v>
       </c>
       <c r="M17" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N17" s="63">
         <v>0.11</v>
@@ -2096,679 +2093,679 @@
     <row r="18" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="50">
-        <f>ROW(B18) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C18" s="57" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D18" s="36" t="s">
-        <v>24</v>
-      </c>
-      <c r="E18" s="37" t="s">
-        <v>48</v>
+        <v>155</v>
+      </c>
+      <c r="E18" s="36" t="s">
+        <v>156</v>
       </c>
       <c r="F18" s="36" t="s">
         <v>65</v>
       </c>
-      <c r="G18" s="37" t="s">
-        <v>81</v>
+      <c r="G18" s="36" t="s">
+        <v>157</v>
       </c>
       <c r="H18" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I18" s="36" t="s">
         <v>99</v>
       </c>
       <c r="J18" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="K18" s="36">
         <v>2</v>
       </c>
       <c r="L18" s="37">
-        <f>K18*5</f>
+        <f t="shared" si="5"/>
         <v>10</v>
       </c>
       <c r="M18" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N18" s="62">
-        <v>0.38</v>
+        <v>0.57799999999999996</v>
       </c>
       <c r="O18" s="62">
         <f t="shared" si="2"/>
-        <v>3.8</v>
+        <v>5.7799999999999994</v>
       </c>
       <c r="P18" s="36"/>
     </row>
     <row r="19" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
-      <c r="C19" s="58" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="67" t="s">
-        <v>25</v>
-      </c>
-      <c r="E19" s="67" t="s">
-        <v>141</v>
-      </c>
-      <c r="F19" s="67" t="s">
-        <v>129</v>
-      </c>
-      <c r="G19" s="67" t="s">
-        <v>142</v>
+      <c r="C19" s="57" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>47</v>
+      </c>
+      <c r="F19" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="G19" s="37" t="s">
+        <v>78</v>
       </c>
       <c r="H19" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="I19" s="67" t="s">
-        <v>143</v>
+        <v>121</v>
+      </c>
+      <c r="I19" s="36" t="s">
+        <v>95</v>
       </c>
       <c r="J19" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="K19" s="38">
-        <v>1</v>
-      </c>
-      <c r="L19" s="39">
-        <f t="shared" ref="L19" si="6">K19*5</f>
-        <v>5</v>
-      </c>
-      <c r="M19" s="68" t="s">
-        <v>144</v>
-      </c>
-      <c r="N19" s="69">
-        <v>3.47</v>
+        <v>121</v>
+      </c>
+      <c r="K19" s="36">
+        <v>2</v>
+      </c>
+      <c r="L19" s="37">
+        <f>K19*5</f>
+        <v>10</v>
+      </c>
+      <c r="M19" s="61" t="s">
+        <v>131</v>
+      </c>
+      <c r="N19" s="62">
+        <v>0.38</v>
       </c>
       <c r="O19" s="62">
         <f t="shared" si="2"/>
-        <v>17.350000000000001</v>
-      </c>
-      <c r="P19" s="38"/>
+        <v>3.8</v>
+      </c>
+      <c r="P19" s="36"/>
     </row>
     <row r="20" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="50">
-        <f>ROW(B20) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="57" t="s">
-        <v>131</v>
-      </c>
-      <c r="D20" s="55" t="s">
-        <v>26</v>
-      </c>
-      <c r="E20" s="59" t="s">
-        <v>49</v>
-      </c>
-      <c r="F20" s="55" t="s">
-        <v>129</v>
-      </c>
-      <c r="G20" s="59" t="s">
+      <c r="C20" s="58" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="67" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" s="67" t="s">
+        <v>137</v>
+      </c>
+      <c r="F20" s="67" t="s">
         <v>125</v>
       </c>
-      <c r="H20" s="55" t="s">
-        <v>125</v>
-      </c>
-      <c r="I20" s="55" t="s">
-        <v>125</v>
-      </c>
-      <c r="J20" s="55" t="s">
-        <v>125</v>
-      </c>
-      <c r="K20" s="55">
+      <c r="G20" s="67" t="s">
+        <v>138</v>
+      </c>
+      <c r="H20" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="I20" s="67" t="s">
+        <v>139</v>
+      </c>
+      <c r="J20" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="K20" s="38">
         <v>1</v>
       </c>
-      <c r="L20" s="59">
-        <f>K20*5</f>
+      <c r="L20" s="39">
+        <f t="shared" ref="L20" si="6">K20*5</f>
         <v>5</v>
       </c>
-      <c r="M20" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="N20" s="64" t="s">
-        <v>125</v>
-      </c>
-      <c r="O20" s="62" t="s">
-        <v>125</v>
-      </c>
-      <c r="P20" s="56" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M20" s="68" t="s">
+        <v>140</v>
+      </c>
+      <c r="N20" s="69">
+        <v>3.47</v>
+      </c>
+      <c r="O20" s="62">
+        <f t="shared" si="2"/>
+        <v>17.350000000000001</v>
+      </c>
+      <c r="P20" s="38"/>
+    </row>
+    <row r="21" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
-      <c r="C21" s="58" t="s">
-        <v>10</v>
-      </c>
-      <c r="D21" s="38" t="s">
-        <v>27</v>
-      </c>
-      <c r="E21" s="39" t="s">
-        <v>50</v>
-      </c>
-      <c r="F21" s="38" t="s">
-        <v>66</v>
-      </c>
-      <c r="G21" s="39" t="s">
-        <v>82</v>
-      </c>
-      <c r="H21" s="38" t="s">
+      <c r="C21" s="57" t="s">
+        <v>127</v>
+      </c>
+      <c r="D21" s="55" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="59" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="55" t="s">
         <v>125</v>
       </c>
-      <c r="I21" s="38" t="s">
-        <v>100</v>
-      </c>
-      <c r="J21" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="K21" s="38">
+      <c r="G21" s="59" t="s">
+        <v>121</v>
+      </c>
+      <c r="H21" s="55" t="s">
+        <v>121</v>
+      </c>
+      <c r="I21" s="55" t="s">
+        <v>121</v>
+      </c>
+      <c r="J21" s="55" t="s">
+        <v>121</v>
+      </c>
+      <c r="K21" s="55">
         <v>1</v>
       </c>
-      <c r="L21" s="39">
-        <f t="shared" ref="L21" si="7">K21*5</f>
+      <c r="L21" s="59">
+        <f>K21*5</f>
         <v>5</v>
       </c>
-      <c r="M21" s="61" t="s">
-        <v>136</v>
-      </c>
-      <c r="N21" s="63" t="s">
-        <v>125</v>
+      <c r="M21" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="N21" s="64" t="s">
+        <v>121</v>
       </c>
       <c r="O21" s="62" t="s">
-        <v>125</v>
-      </c>
-      <c r="P21" s="38"/>
-    </row>
-    <row r="22" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>121</v>
+      </c>
+      <c r="P21" s="56" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="50">
-        <f>ROW(B22) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C22" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="D22" s="36" t="s">
+      <c r="D22" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22" s="39" t="s">
+        <v>49</v>
+      </c>
+      <c r="F22" s="38" t="s">
+        <v>64</v>
+      </c>
+      <c r="G22" s="39" t="s">
+        <v>79</v>
+      </c>
+      <c r="H22" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="I22" s="38" t="s">
+        <v>96</v>
+      </c>
+      <c r="J22" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="K22" s="38">
+        <v>1</v>
+      </c>
+      <c r="L22" s="39">
+        <f t="shared" ref="L22" si="7">K22*5</f>
+        <v>5</v>
+      </c>
+      <c r="M22" s="61" t="s">
+        <v>132</v>
+      </c>
+      <c r="N22" s="63" t="s">
+        <v>121</v>
+      </c>
+      <c r="O22" s="62" t="s">
+        <v>121</v>
+      </c>
+      <c r="P22" s="38"/>
+    </row>
+    <row r="23" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="1"/>
+      <c r="B23" s="50">
+        <f>ROW(B23) - ROW($B$9)</f>
+        <v>14</v>
+      </c>
+      <c r="C23" s="58" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="E22" s="37" t="s">
-        <v>51</v>
-      </c>
-      <c r="F22" s="36" t="s">
-        <v>67</v>
-      </c>
-      <c r="G22" s="37" t="s">
-        <v>83</v>
-      </c>
-      <c r="H22" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="I22" s="36" t="s">
-        <v>101</v>
-      </c>
-      <c r="J22" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="K22" s="36">
+      <c r="E23" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="F23" s="36" t="s">
+        <v>65</v>
+      </c>
+      <c r="G23" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="H23" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="I23" s="36" t="s">
+        <v>97</v>
+      </c>
+      <c r="J23" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="K23" s="36">
         <v>1</v>
       </c>
-      <c r="L22" s="37">
-        <f>K22*5</f>
+      <c r="L23" s="37">
+        <f>K23*5</f>
         <v>5</v>
       </c>
-      <c r="M22" s="61" t="s">
-        <v>135</v>
-      </c>
-      <c r="N22" s="62">
+      <c r="M23" s="61" t="s">
+        <v>131</v>
+      </c>
+      <c r="N23" s="62">
         <v>0.46</v>
       </c>
-      <c r="O22" s="62">
+      <c r="O23" s="62">
         <f t="shared" si="2"/>
         <v>2.3000000000000003</v>
       </c>
-      <c r="P22" s="36"/>
-    </row>
-    <row r="23" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="1"/>
-      <c r="B23" s="50">
+      <c r="P23" s="36"/>
+    </row>
+    <row r="24" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="1"/>
+      <c r="B24" s="50">
         <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="C23" s="58" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="38" t="s">
+      <c r="D24" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="E23" s="39" t="s">
-        <v>52</v>
-      </c>
-      <c r="F23" s="38" t="s">
-        <v>68</v>
-      </c>
-      <c r="G23" s="39" t="s">
-        <v>84</v>
-      </c>
-      <c r="H23" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="I23" s="38" t="s">
-        <v>95</v>
-      </c>
-      <c r="J23" s="38" t="s">
-        <v>113</v>
-      </c>
-      <c r="K23" s="38">
+      <c r="E24" s="39" t="s">
+        <v>51</v>
+      </c>
+      <c r="F24" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="G24" s="39" t="s">
+        <v>81</v>
+      </c>
+      <c r="H24" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="I24" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="J24" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="K24" s="38">
         <v>1</v>
       </c>
-      <c r="L23" s="39">
-        <f t="shared" ref="L23" si="8">K23*5</f>
+      <c r="L24" s="39">
+        <f t="shared" ref="L24" si="8">K24*5</f>
         <v>5</v>
       </c>
-      <c r="M23" s="61" t="s">
-        <v>135</v>
-      </c>
-      <c r="N23" s="63">
+      <c r="M24" s="61" t="s">
+        <v>131</v>
+      </c>
+      <c r="N24" s="63">
         <v>0.1</v>
       </c>
-      <c r="O23" s="62">
+      <c r="O24" s="62">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="P23" s="38"/>
-    </row>
-    <row r="24" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="1"/>
-      <c r="B24" s="50">
-        <f>ROW(B24) - ROW($B$9)</f>
-        <v>15</v>
-      </c>
-      <c r="C24" s="57" t="s">
+      <c r="P24" s="38"/>
+    </row>
+    <row r="25" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="1"/>
+      <c r="B25" s="50">
+        <f>ROW(B25) - ROW($B$9)</f>
+        <v>16</v>
+      </c>
+      <c r="C25" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="36" t="s">
-        <v>148</v>
-      </c>
-      <c r="E24" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="F24" s="36" t="s">
-        <v>146</v>
-      </c>
-      <c r="G24" s="36" t="s">
-        <v>147</v>
-      </c>
-      <c r="H24" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="I24" s="36" t="s">
-        <v>95</v>
-      </c>
-      <c r="J24" s="36" t="s">
-        <v>114</v>
-      </c>
-      <c r="K24" s="36">
+      <c r="D25" s="36" t="s">
+        <v>144</v>
+      </c>
+      <c r="E25" s="36" t="s">
+        <v>141</v>
+      </c>
+      <c r="F25" s="36" t="s">
+        <v>142</v>
+      </c>
+      <c r="G25" s="36" t="s">
+        <v>143</v>
+      </c>
+      <c r="H25" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="I25" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="J25" s="36" t="s">
+        <v>110</v>
+      </c>
+      <c r="K25" s="36">
         <v>12</v>
       </c>
-      <c r="L24" s="37">
-        <f>K24*5</f>
+      <c r="L25" s="37">
+        <f>K25*5</f>
         <v>60</v>
       </c>
-      <c r="M24" s="61" t="s">
-        <v>135</v>
-      </c>
-      <c r="N24" s="63">
+      <c r="M25" s="61" t="s">
+        <v>131</v>
+      </c>
+      <c r="N25" s="63">
         <v>0.1</v>
       </c>
-      <c r="O24" s="62">
+      <c r="O25" s="62">
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="P24" s="36"/>
-    </row>
-    <row r="25" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="1"/>
-      <c r="B25" s="50">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="C25" s="58" t="s">
-        <v>11</v>
-      </c>
-      <c r="D25" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E25" s="39" t="s">
-        <v>53</v>
-      </c>
-      <c r="F25" s="38" t="s">
-        <v>68</v>
-      </c>
-      <c r="G25" s="39" t="s">
-        <v>85</v>
-      </c>
-      <c r="H25" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="I25" s="38" t="s">
-        <v>95</v>
-      </c>
-      <c r="J25" s="38" t="s">
-        <v>115</v>
-      </c>
-      <c r="K25" s="38">
-        <v>3</v>
-      </c>
-      <c r="L25" s="39">
-        <f t="shared" ref="L25" si="9">K25*5</f>
-        <v>15</v>
-      </c>
-      <c r="M25" s="61" t="s">
-        <v>135</v>
-      </c>
-      <c r="N25" s="63">
-        <v>0.1</v>
-      </c>
-      <c r="O25" s="62">
-        <f t="shared" si="2"/>
-        <v>1.5</v>
-      </c>
-      <c r="P25" s="38"/>
+      <c r="P25" s="36"/>
     </row>
     <row r="26" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="50">
-        <f>ROW(B26) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="57" t="s">
+      <c r="C26" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="D26" s="36" t="s">
-        <v>30</v>
-      </c>
-      <c r="E26" s="37" t="s">
-        <v>54</v>
-      </c>
-      <c r="F26" s="36" t="s">
-        <v>68</v>
-      </c>
-      <c r="G26" s="37" t="s">
-        <v>86</v>
-      </c>
-      <c r="H26" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="I26" s="36" t="s">
-        <v>95</v>
-      </c>
-      <c r="J26" s="36" t="s">
-        <v>116</v>
-      </c>
-      <c r="K26" s="36">
-        <v>4</v>
-      </c>
-      <c r="L26" s="37">
-        <f>K26*5</f>
-        <v>20</v>
+      <c r="D26" s="38" t="s">
+        <v>145</v>
+      </c>
+      <c r="E26" s="39" t="s">
+        <v>52</v>
+      </c>
+      <c r="F26" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="G26" s="39" t="s">
+        <v>82</v>
+      </c>
+      <c r="H26" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="I26" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="J26" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="K26" s="38">
+        <v>3</v>
+      </c>
+      <c r="L26" s="39">
+        <f t="shared" ref="L26" si="9">K26*5</f>
+        <v>15</v>
       </c>
       <c r="M26" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N26" s="63">
         <v>0.1</v>
       </c>
       <c r="O26" s="62">
         <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="P26" s="36"/>
+        <v>1.5</v>
+      </c>
+      <c r="P26" s="38"/>
     </row>
     <row r="27" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
-      <c r="C27" s="58" t="s">
+      <c r="C27" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="D27" s="38" t="s">
-        <v>31</v>
-      </c>
-      <c r="E27" s="39" t="s">
-        <v>55</v>
-      </c>
-      <c r="F27" s="38" t="s">
-        <v>68</v>
-      </c>
-      <c r="G27" s="39" t="s">
-        <v>87</v>
-      </c>
-      <c r="H27" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="I27" s="38" t="s">
-        <v>95</v>
-      </c>
-      <c r="J27" s="38" t="s">
-        <v>117</v>
-      </c>
-      <c r="K27" s="38">
-        <v>1</v>
-      </c>
-      <c r="L27" s="39">
-        <f t="shared" ref="L27" si="10">K27*5</f>
-        <v>5</v>
+      <c r="D27" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="F27" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="G27" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="H27" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="I27" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="J27" s="36" t="s">
+        <v>112</v>
+      </c>
+      <c r="K27" s="36">
+        <v>4</v>
+      </c>
+      <c r="L27" s="37">
+        <f>K27*5</f>
+        <v>20</v>
       </c>
       <c r="M27" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N27" s="63">
         <v>0.1</v>
       </c>
       <c r="O27" s="62">
         <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="P27" s="38"/>
+        <v>2</v>
+      </c>
+      <c r="P27" s="36"/>
     </row>
     <row r="28" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="50">
-        <f>ROW(B28) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C28" s="57" t="s">
+      <c r="C28" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="D28" s="36" t="s">
-        <v>32</v>
-      </c>
-      <c r="E28" s="37" t="s">
-        <v>56</v>
-      </c>
-      <c r="F28" s="36" t="s">
-        <v>68</v>
-      </c>
-      <c r="G28" s="37" t="s">
-        <v>88</v>
-      </c>
-      <c r="H28" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="I28" s="36" t="s">
-        <v>95</v>
-      </c>
-      <c r="J28" s="36" t="s">
-        <v>118</v>
-      </c>
-      <c r="K28" s="36">
-        <v>4</v>
-      </c>
-      <c r="L28" s="37">
-        <f>K28*5</f>
-        <v>20</v>
+      <c r="D28" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="E28" s="39" t="s">
+        <v>54</v>
+      </c>
+      <c r="F28" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="G28" s="39" t="s">
+        <v>84</v>
+      </c>
+      <c r="H28" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="I28" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="J28" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="K28" s="38">
+        <v>1</v>
+      </c>
+      <c r="L28" s="39">
+        <f t="shared" ref="L28" si="10">K28*5</f>
+        <v>5</v>
       </c>
       <c r="M28" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N28" s="63">
         <v>0.1</v>
       </c>
       <c r="O28" s="62">
         <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="P28" s="36"/>
+        <v>0.5</v>
+      </c>
+      <c r="P28" s="38"/>
     </row>
     <row r="29" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B29) - ROW($B$9)</f>
         <v>20</v>
       </c>
-      <c r="C29" s="58" t="s">
+      <c r="C29" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="D29" s="38" t="s">
-        <v>33</v>
-      </c>
-      <c r="E29" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="F29" s="38" t="s">
-        <v>68</v>
-      </c>
-      <c r="G29" s="39" t="s">
-        <v>89</v>
-      </c>
-      <c r="H29" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="I29" s="38" t="s">
-        <v>95</v>
-      </c>
-      <c r="J29" s="38" t="s">
-        <v>119</v>
-      </c>
-      <c r="K29" s="38">
-        <v>2</v>
-      </c>
-      <c r="L29" s="39">
-        <f t="shared" ref="L29" si="11">K29*5</f>
-        <v>10</v>
+      <c r="D29" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="E29" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="F29" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="G29" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="H29" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="I29" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="J29" s="36" t="s">
+        <v>114</v>
+      </c>
+      <c r="K29" s="36">
+        <v>4</v>
+      </c>
+      <c r="L29" s="37">
+        <f>K29*5</f>
+        <v>20</v>
       </c>
       <c r="M29" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N29" s="63">
         <v>0.1</v>
       </c>
       <c r="O29" s="62">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="P29" s="38"/>
+        <v>2</v>
+      </c>
+      <c r="P29" s="36"/>
     </row>
     <row r="30" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="50">
-        <f>ROW(B30) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C30" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="D30" s="36" t="s">
-        <v>34</v>
-      </c>
-      <c r="E30" s="37" t="s">
-        <v>58</v>
-      </c>
-      <c r="F30" s="36" t="s">
-        <v>68</v>
-      </c>
-      <c r="G30" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="H30" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="I30" s="36" t="s">
-        <v>95</v>
-      </c>
-      <c r="J30" s="36" t="s">
-        <v>120</v>
-      </c>
-      <c r="K30" s="36">
-        <v>1</v>
-      </c>
-      <c r="L30" s="37">
-        <f>K30*5</f>
-        <v>5</v>
+      <c r="D30" s="38" t="s">
+        <v>33</v>
+      </c>
+      <c r="E30" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="F30" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="G30" s="39" t="s">
+        <v>86</v>
+      </c>
+      <c r="H30" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="I30" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="J30" s="38" t="s">
+        <v>115</v>
+      </c>
+      <c r="K30" s="38">
+        <v>2</v>
+      </c>
+      <c r="L30" s="39">
+        <f t="shared" ref="L30" si="11">K30*5</f>
+        <v>10</v>
       </c>
       <c r="M30" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N30" s="63">
         <v>0.1</v>
       </c>
       <c r="O30" s="62">
         <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="P30" s="36"/>
+        <v>1</v>
+      </c>
+      <c r="P30" s="38"/>
     </row>
     <row r="31" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B31) - ROW($B$9)</f>
         <v>22</v>
       </c>
       <c r="C31" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="D31" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="E31" s="39" t="s">
-        <v>59</v>
-      </c>
-      <c r="F31" s="38" t="s">
-        <v>68</v>
-      </c>
-      <c r="G31" s="39" t="s">
+      <c r="D31" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="E31" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="F31" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="G31" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="H31" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="I31" s="36" t="s">
         <v>91</v>
       </c>
-      <c r="H31" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="I31" s="38" t="s">
-        <v>95</v>
-      </c>
-      <c r="J31" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="K31" s="38">
+      <c r="J31" s="36" t="s">
+        <v>116</v>
+      </c>
+      <c r="K31" s="36">
         <v>1</v>
       </c>
-      <c r="L31" s="39">
-        <f t="shared" ref="L31:L32" si="12">K31*5</f>
+      <c r="L31" s="37">
+        <f>K31*5</f>
         <v>5</v>
       </c>
       <c r="M31" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N31" s="63">
         <v>0.1</v>
@@ -2777,7 +2774,7 @@
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="P31" s="38"/>
+      <c r="P31" s="36"/>
     </row>
     <row r="32" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
@@ -2785,146 +2782,146 @@
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C32" s="57" t="s">
+      <c r="C32" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="D32" s="36" t="s">
-        <v>150</v>
-      </c>
-      <c r="E32" s="36" t="s">
-        <v>151</v>
-      </c>
-      <c r="F32" s="36" t="s">
-        <v>152</v>
-      </c>
-      <c r="G32" s="36" t="s">
-        <v>153</v>
-      </c>
-      <c r="H32" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="I32" s="36" t="s">
-        <v>95</v>
-      </c>
-      <c r="J32" s="36" t="s">
-        <v>154</v>
-      </c>
-      <c r="K32" s="36">
+      <c r="D32" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="E32" s="39" t="s">
+        <v>58</v>
+      </c>
+      <c r="F32" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="G32" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="H32" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="I32" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="J32" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="K32" s="38">
         <v>1</v>
       </c>
       <c r="L32" s="39">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="L32:L33" si="12">K32*5</f>
         <v>5</v>
       </c>
       <c r="M32" s="61" t="s">
-        <v>135</v>
-      </c>
-      <c r="N32" s="62">
+        <v>131</v>
+      </c>
+      <c r="N32" s="63">
         <v>0.1</v>
       </c>
       <c r="O32" s="62">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="P32" s="36"/>
+      <c r="P32" s="38"/>
     </row>
     <row r="33" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="50">
-        <f>ROW(B33) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C33" s="57" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D33" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="E33" s="37" t="s">
-        <v>60</v>
+        <v>146</v>
+      </c>
+      <c r="E33" s="36" t="s">
+        <v>147</v>
       </c>
       <c r="F33" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="G33" s="37" t="s">
-        <v>92</v>
+        <v>148</v>
+      </c>
+      <c r="G33" s="36" t="s">
+        <v>149</v>
       </c>
       <c r="H33" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I33" s="36" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="J33" s="36" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="K33" s="36">
         <v>1</v>
       </c>
-      <c r="L33" s="37">
-        <f>K33*5</f>
+      <c r="L33" s="39">
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="M33" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N33" s="62">
-        <v>3.85</v>
+        <v>0.1</v>
       </c>
       <c r="O33" s="62">
         <f t="shared" si="2"/>
-        <v>19.25</v>
+        <v>0.5</v>
       </c>
       <c r="P33" s="36"/>
     </row>
     <row r="34" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="58" t="s">
-        <v>13</v>
-      </c>
-      <c r="D34" s="38" t="s">
-        <v>37</v>
-      </c>
-      <c r="E34" s="39" t="s">
-        <v>61</v>
-      </c>
-      <c r="F34" s="38" t="s">
-        <v>70</v>
-      </c>
-      <c r="G34" s="39" t="s">
-        <v>93</v>
-      </c>
-      <c r="H34" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="I34" s="38" t="s">
-        <v>103</v>
-      </c>
-      <c r="J34" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="K34" s="38">
+      <c r="C34" s="57" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="F34" s="36" t="s">
+        <v>67</v>
+      </c>
+      <c r="G34" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="H34" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="I34" s="36" t="s">
+        <v>98</v>
+      </c>
+      <c r="J34" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="K34" s="36">
         <v>1</v>
       </c>
-      <c r="L34" s="39">
-        <f t="shared" ref="L34" si="13">K34*5</f>
+      <c r="L34" s="37">
+        <f>K34*5</f>
         <v>5</v>
       </c>
       <c r="M34" s="61" t="s">
-        <v>135</v>
-      </c>
-      <c r="N34" s="63">
-        <v>0.87</v>
+        <v>131</v>
+      </c>
+      <c r="N34" s="62">
+        <v>3.85</v>
       </c>
       <c r="O34" s="62">
         <f t="shared" si="2"/>
-        <v>4.3499999999999996</v>
-      </c>
-      <c r="P34" s="38"/>
+        <v>19.25</v>
+      </c>
+      <c r="P34" s="36"/>
     </row>
     <row r="35" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
@@ -2936,25 +2933,25 @@
         <v>14</v>
       </c>
       <c r="D35" s="36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E35" s="37" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F35" s="36" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G35" s="37" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="H35" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I35" s="36" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="J35" s="36" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="K35" s="36">
         <v>1</v>
@@ -2964,7 +2961,7 @@
         <v>5</v>
       </c>
       <c r="M35" s="61" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="N35" s="62">
         <v>0.59</v>
@@ -2982,43 +2979,43 @@
         <v>27</v>
       </c>
       <c r="C36" s="57" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D36" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E36" s="36" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="G36" s="36" t="s">
-        <v>157</v>
-      </c>
-      <c r="H36" s="75"/>
+        <v>153</v>
+      </c>
+      <c r="H36" s="70"/>
       <c r="I36" s="36" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="J36" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="K36" s="36">
         <v>1</v>
       </c>
-      <c r="L36" s="75">
+      <c r="L36" s="70">
         <v>5</v>
       </c>
       <c r="M36" s="61" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="N36" s="63" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="O36" s="62" t="s">
-        <v>125</v>
-      </c>
-      <c r="P36" s="76"/>
+        <v>121</v>
+      </c>
+      <c r="P36" s="71"/>
     </row>
     <row r="37" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
@@ -3032,14 +3029,14 @@
       <c r="I37" s="34"/>
       <c r="J37" s="35"/>
       <c r="K37" s="35"/>
-      <c r="L37" s="73" t="s">
-        <v>137</v>
-      </c>
-      <c r="M37" s="74"/>
-      <c r="N37" s="74"/>
+      <c r="L37" s="75" t="s">
+        <v>133</v>
+      </c>
+      <c r="M37" s="76"/>
+      <c r="N37" s="76"/>
       <c r="O37" s="65">
         <f>SUM(O10:O35)</f>
-        <v>86.97</v>
+        <v>88.4</v>
       </c>
       <c r="P37" s="41"/>
     </row>
@@ -3055,14 +3052,14 @@
       <c r="I38" s="9"/>
       <c r="J38" s="9"/>
       <c r="K38" s="9"/>
-      <c r="L38" s="73" t="s">
-        <v>138</v>
-      </c>
-      <c r="M38" s="74"/>
-      <c r="N38" s="74"/>
+      <c r="L38" s="75" t="s">
+        <v>134</v>
+      </c>
+      <c r="M38" s="76"/>
+      <c r="N38" s="76"/>
       <c r="O38" s="66">
         <f>O37/5</f>
-        <v>17.393999999999998</v>
+        <v>17.68</v>
       </c>
       <c r="P38" s="42"/>
     </row>
@@ -3081,22 +3078,22 @@
     <hyperlink ref="M15" r:id="rId5"/>
     <hyperlink ref="M16" r:id="rId6"/>
     <hyperlink ref="M17" r:id="rId7"/>
-    <hyperlink ref="M18" r:id="rId8"/>
-    <hyperlink ref="M22" r:id="rId9"/>
-    <hyperlink ref="M23" r:id="rId10"/>
-    <hyperlink ref="M25" r:id="rId11"/>
-    <hyperlink ref="M26" r:id="rId12"/>
-    <hyperlink ref="M27" r:id="rId13"/>
-    <hyperlink ref="M28" r:id="rId14"/>
-    <hyperlink ref="M29" r:id="rId15"/>
-    <hyperlink ref="M30" r:id="rId16"/>
-    <hyperlink ref="M31" r:id="rId17"/>
-    <hyperlink ref="M33" r:id="rId18"/>
-    <hyperlink ref="M34" r:id="rId19"/>
-    <hyperlink ref="M35" r:id="rId20"/>
-    <hyperlink ref="M19" r:id="rId21"/>
-    <hyperlink ref="M24" r:id="rId22"/>
-    <hyperlink ref="M32" r:id="rId23"/>
+    <hyperlink ref="M19" r:id="rId8"/>
+    <hyperlink ref="M23" r:id="rId9"/>
+    <hyperlink ref="M24" r:id="rId10"/>
+    <hyperlink ref="M26" r:id="rId11"/>
+    <hyperlink ref="M27" r:id="rId12"/>
+    <hyperlink ref="M28" r:id="rId13"/>
+    <hyperlink ref="M29" r:id="rId14"/>
+    <hyperlink ref="M30" r:id="rId15"/>
+    <hyperlink ref="M31" r:id="rId16"/>
+    <hyperlink ref="M32" r:id="rId17"/>
+    <hyperlink ref="M34" r:id="rId18"/>
+    <hyperlink ref="M35" r:id="rId19"/>
+    <hyperlink ref="M20" r:id="rId20"/>
+    <hyperlink ref="M25" r:id="rId21"/>
+    <hyperlink ref="M33" r:id="rId22"/>
+    <hyperlink ref="M18" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId24"/>

</xml_diff>

<commit_message>
#17 Final Client BOM
</commit_message>
<xml_diff>
--- a/Design Files/Ethernet-Module-v2.0/BOM/Client_BOM_Ethernet-Module-v2.0.xlsx
+++ b/Design Files/Ethernet-Module-v2.0/BOM/Client_BOM_Ethernet-Module-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="150">
   <si>
     <t>Component list</t>
   </si>
@@ -405,27 +405,6 @@
     <t xml:space="preserve">Mini PCIe SMD Pad </t>
   </si>
   <si>
-    <t>Unit Cost (5 Boards)</t>
-  </si>
-  <si>
-    <t>Total Cost (5 Boards)</t>
-  </si>
-  <si>
-    <t>Links</t>
-  </si>
-  <si>
-    <t>Digikey</t>
-  </si>
-  <si>
-    <t>Custom Supplier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Component Cost </t>
-  </si>
-  <si>
-    <t>Single Board Cost</t>
-  </si>
-  <si>
     <t>Bill of Materials for Project [Ethernet-Module-v2.0.]</t>
   </si>
   <si>
@@ -439,9 +418,6 @@
   </si>
   <si>
     <t>Abracon</t>
-  </si>
-  <si>
-    <t>Mouser</t>
   </si>
   <si>
     <t>RES SMD 10K OHM 1% 1/20W 0201</t>
@@ -499,12 +475,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -653,14 +627,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="14"/>
       <name val="Calibri"/>
@@ -694,7 +660,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -902,25 +868,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1080,39 +1032,15 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1123,17 +1051,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1159,13 +1078,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>19942</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>1905000</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>171450</xdr:rowOff>
@@ -1473,7 +1392,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P38"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1487,12 +1406,11 @@
     <col min="10" max="10" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.140625" customWidth="1"/>
-    <col min="14" max="15" width="18.28515625" customWidth="1"/>
-    <col min="16" max="16" width="29.42578125" customWidth="1"/>
+    <col min="13" max="13" width="29.42578125" customWidth="1"/>
+    <col min="15" max="15" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1502,15 +1420,12 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="72"/>
-      <c r="P1" s="72"/>
-    </row>
-    <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+    </row>
+    <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="43"/>
@@ -1519,7 +1434,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -1527,12 +1442,9 @@
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="40"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M2" s="40"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="44"/>
@@ -1541,7 +1453,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -1549,12 +1461,9 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="73"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M3" s="64"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="44"/>
@@ -1563,7 +1472,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1571,12 +1480,9 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="60"/>
-      <c r="N4" s="60"/>
-      <c r="O4" s="60"/>
-      <c r="P4" s="74"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M4" s="65"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="44"/>
@@ -1593,12 +1499,9 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="60"/>
-      <c r="N5" s="60"/>
-      <c r="O5" s="60"/>
-      <c r="P5" s="74"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M5" s="65"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="45"/>
@@ -1611,12 +1514,9 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="60"/>
-      <c r="N6" s="60"/>
-      <c r="O6" s="60"/>
-      <c r="P6" s="74"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M6" s="65"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="46"/>
@@ -1629,12 +1529,9 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="74"/>
-    </row>
-    <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M7" s="65"/>
+    </row>
+    <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="47"/>
@@ -1647,12 +1544,9 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="74"/>
-    </row>
-    <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M8" s="65"/>
+    </row>
+    <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
@@ -1688,19 +1582,10 @@
         <v>123</v>
       </c>
       <c r="M9" s="29" t="s">
-        <v>130</v>
-      </c>
-      <c r="N9" s="29" t="s">
-        <v>128</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>129</v>
-      </c>
-      <c r="P9" s="29" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="50">
         <f>ROW(B10) - ROW($B$9)</f>
@@ -1737,19 +1622,9 @@
         <f>K10*5</f>
         <v>10</v>
       </c>
-      <c r="M10" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N10" s="62">
-        <v>0.68</v>
-      </c>
-      <c r="O10" s="62">
-        <f>N10*L10</f>
-        <v>6.8000000000000007</v>
-      </c>
-      <c r="P10" s="36"/>
-    </row>
-    <row r="11" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M10" s="36"/>
+    </row>
+    <row r="11" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="50">
         <f t="shared" ref="B11:B33" si="0">ROW(B11) - ROW($B$9)</f>
@@ -1786,19 +1661,9 @@
         <f t="shared" ref="L11" si="1">K11*5</f>
         <v>35</v>
       </c>
-      <c r="M11" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N11" s="63">
-        <v>0.1</v>
-      </c>
-      <c r="O11" s="62">
-        <f t="shared" ref="O11:O35" si="2">N11*L11</f>
-        <v>3.5</v>
-      </c>
-      <c r="P11" s="38"/>
-    </row>
-    <row r="12" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M11" s="38"/>
+    </row>
+    <row r="12" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="50">
         <f>ROW(B12) - ROW($B$9)</f>
@@ -1835,19 +1700,9 @@
         <f>K12*5</f>
         <v>10</v>
       </c>
-      <c r="M12" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N12" s="62">
-        <v>0.75</v>
-      </c>
-      <c r="O12" s="62">
-        <f t="shared" si="2"/>
-        <v>7.5</v>
-      </c>
-      <c r="P12" s="36"/>
-    </row>
-    <row r="13" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M12" s="36"/>
+    </row>
+    <row r="13" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="50">
         <f t="shared" si="0"/>
@@ -1881,20 +1736,12 @@
         <v>2</v>
       </c>
       <c r="L13" s="39">
-        <f t="shared" ref="L13" si="3">K13*5</f>
+        <f t="shared" ref="L13" si="2">K13*5</f>
         <v>10</v>
       </c>
-      <c r="M13" s="61" t="s">
-        <v>132</v>
-      </c>
-      <c r="N13" s="63"/>
-      <c r="O13" s="62">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P13" s="38"/>
-    </row>
-    <row r="14" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M13" s="38"/>
+    </row>
+    <row r="14" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="50">
         <f>ROW(B14) - ROW($B$9)</f>
@@ -1931,19 +1778,9 @@
         <f>K14*5</f>
         <v>5</v>
       </c>
-      <c r="M14" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N14" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="O14" s="62">
-        <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="P14" s="36"/>
-    </row>
-    <row r="15" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M14" s="36"/>
+    </row>
+    <row r="15" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="50">
         <f t="shared" si="0"/>
@@ -1977,22 +1814,12 @@
         <v>2</v>
       </c>
       <c r="L15" s="39">
-        <f t="shared" ref="L15" si="4">K15*5</f>
+        <f t="shared" ref="L15" si="3">K15*5</f>
         <v>10</v>
       </c>
-      <c r="M15" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N15" s="63">
-        <v>9.7000000000000003E-2</v>
-      </c>
-      <c r="O15" s="62">
-        <f t="shared" si="2"/>
-        <v>0.97</v>
-      </c>
-      <c r="P15" s="38"/>
-    </row>
-    <row r="16" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M15" s="38"/>
+    </row>
+    <row r="16" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="50">
         <f>ROW(B16) - ROW($B$9)</f>
@@ -2029,19 +1856,9 @@
         <f>K16*5</f>
         <v>5</v>
       </c>
-      <c r="M16" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N16" s="62">
-        <v>0.32</v>
-      </c>
-      <c r="O16" s="62">
-        <f t="shared" si="2"/>
-        <v>1.6</v>
-      </c>
-      <c r="P16" s="36"/>
-    </row>
-    <row r="17" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M16" s="36"/>
+    </row>
+    <row r="17" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="50">
         <f t="shared" si="0"/>
@@ -2075,22 +1892,12 @@
         <v>2</v>
       </c>
       <c r="L17" s="39">
-        <f t="shared" ref="L17:L18" si="5">K17*5</f>
+        <f t="shared" ref="L17:L18" si="4">K17*5</f>
         <v>10</v>
       </c>
-      <c r="M17" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N17" s="63">
-        <v>0.11</v>
-      </c>
-      <c r="O17" s="62">
-        <f t="shared" si="2"/>
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="P17" s="38"/>
-    </row>
-    <row r="18" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M17" s="38"/>
+    </row>
+    <row r="18" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="50">
         <f t="shared" si="0"/>
@@ -2100,16 +1907,16 @@
         <v>13</v>
       </c>
       <c r="D18" s="36" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="E18" s="36" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="F18" s="36" t="s">
         <v>65</v>
       </c>
       <c r="G18" s="36" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="H18" s="36" t="s">
         <v>121</v>
@@ -2124,22 +1931,12 @@
         <v>2</v>
       </c>
       <c r="L18" s="37">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="M18" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N18" s="62">
-        <v>0.57799999999999996</v>
-      </c>
-      <c r="O18" s="62">
-        <f t="shared" si="2"/>
-        <v>5.7799999999999994</v>
-      </c>
-      <c r="P18" s="36"/>
-    </row>
-    <row r="19" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M18" s="36"/>
+    </row>
+    <row r="19" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="50">
         <f>ROW(B19) - ROW($B$9)</f>
@@ -2176,19 +1973,9 @@
         <f>K19*5</f>
         <v>10</v>
       </c>
-      <c r="M19" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N19" s="62">
-        <v>0.38</v>
-      </c>
-      <c r="O19" s="62">
-        <f t="shared" si="2"/>
-        <v>3.8</v>
-      </c>
-      <c r="P19" s="36"/>
-    </row>
-    <row r="20" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M19" s="36"/>
+    </row>
+    <row r="20" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="50">
         <f t="shared" si="0"/>
@@ -2197,23 +1984,23 @@
       <c r="C20" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="D20" s="67" t="s">
+      <c r="D20" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="67" t="s">
-        <v>137</v>
-      </c>
-      <c r="F20" s="67" t="s">
+      <c r="E20" s="60" t="s">
+        <v>130</v>
+      </c>
+      <c r="F20" s="60" t="s">
         <v>125</v>
       </c>
-      <c r="G20" s="67" t="s">
-        <v>138</v>
+      <c r="G20" s="60" t="s">
+        <v>131</v>
       </c>
       <c r="H20" s="36" t="s">
         <v>121</v>
       </c>
-      <c r="I20" s="67" t="s">
-        <v>139</v>
+      <c r="I20" s="60" t="s">
+        <v>132</v>
       </c>
       <c r="J20" s="36" t="s">
         <v>121</v>
@@ -2222,22 +2009,12 @@
         <v>1</v>
       </c>
       <c r="L20" s="39">
-        <f t="shared" ref="L20" si="6">K20*5</f>
+        <f t="shared" ref="L20" si="5">K20*5</f>
         <v>5</v>
       </c>
-      <c r="M20" s="68" t="s">
-        <v>140</v>
-      </c>
-      <c r="N20" s="69">
-        <v>3.47</v>
-      </c>
-      <c r="O20" s="62">
-        <f t="shared" si="2"/>
-        <v>17.350000000000001</v>
-      </c>
-      <c r="P20" s="38"/>
-    </row>
-    <row r="21" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M20" s="38"/>
+    </row>
+    <row r="21" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="50">
         <f>ROW(B21) - ROW($B$9)</f>
@@ -2274,20 +2051,11 @@
         <f>K21*5</f>
         <v>5</v>
       </c>
-      <c r="M21" s="36" t="s">
-        <v>121</v>
-      </c>
-      <c r="N21" s="64" t="s">
-        <v>121</v>
-      </c>
-      <c r="O21" s="62" t="s">
-        <v>121</v>
-      </c>
-      <c r="P21" s="56" t="s">
+      <c r="M21" s="56" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="50">
         <f t="shared" si="0"/>
@@ -2321,21 +2089,12 @@
         <v>1</v>
       </c>
       <c r="L22" s="39">
-        <f t="shared" ref="L22" si="7">K22*5</f>
+        <f t="shared" ref="L22" si="6">K22*5</f>
         <v>5</v>
       </c>
-      <c r="M22" s="61" t="s">
-        <v>132</v>
-      </c>
-      <c r="N22" s="63" t="s">
-        <v>121</v>
-      </c>
-      <c r="O22" s="62" t="s">
-        <v>121</v>
-      </c>
-      <c r="P22" s="38"/>
-    </row>
-    <row r="23" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M22" s="38"/>
+    </row>
+    <row r="23" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="50">
         <f>ROW(B23) - ROW($B$9)</f>
@@ -2372,19 +2131,9 @@
         <f>K23*5</f>
         <v>5</v>
       </c>
-      <c r="M23" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N23" s="62">
-        <v>0.46</v>
-      </c>
-      <c r="O23" s="62">
-        <f t="shared" si="2"/>
-        <v>2.3000000000000003</v>
-      </c>
-      <c r="P23" s="36"/>
-    </row>
-    <row r="24" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M23" s="36"/>
+    </row>
+    <row r="24" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="50">
         <f t="shared" si="0"/>
@@ -2418,22 +2167,12 @@
         <v>1</v>
       </c>
       <c r="L24" s="39">
-        <f t="shared" ref="L24" si="8">K24*5</f>
+        <f t="shared" ref="L24" si="7">K24*5</f>
         <v>5</v>
       </c>
-      <c r="M24" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N24" s="63">
-        <v>0.1</v>
-      </c>
-      <c r="O24" s="62">
-        <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="P24" s="38"/>
-    </row>
-    <row r="25" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M24" s="38"/>
+    </row>
+    <row r="25" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="50">
         <f>ROW(B25) - ROW($B$9)</f>
@@ -2443,16 +2182,16 @@
         <v>11</v>
       </c>
       <c r="D25" s="36" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="E25" s="36" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="F25" s="36" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="G25" s="36" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="H25" s="36" t="s">
         <v>121</v>
@@ -2470,19 +2209,9 @@
         <f>K25*5</f>
         <v>60</v>
       </c>
-      <c r="M25" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N25" s="63">
-        <v>0.1</v>
-      </c>
-      <c r="O25" s="62">
-        <f t="shared" si="2"/>
-        <v>6</v>
-      </c>
-      <c r="P25" s="36"/>
-    </row>
-    <row r="26" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M25" s="36"/>
+    </row>
+    <row r="26" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="50">
         <f t="shared" si="0"/>
@@ -2492,7 +2221,7 @@
         <v>11</v>
       </c>
       <c r="D26" s="38" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="E26" s="39" t="s">
         <v>52</v>
@@ -2516,22 +2245,12 @@
         <v>3</v>
       </c>
       <c r="L26" s="39">
-        <f t="shared" ref="L26" si="9">K26*5</f>
+        <f t="shared" ref="L26" si="8">K26*5</f>
         <v>15</v>
       </c>
-      <c r="M26" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N26" s="63">
-        <v>0.1</v>
-      </c>
-      <c r="O26" s="62">
-        <f t="shared" si="2"/>
-        <v>1.5</v>
-      </c>
-      <c r="P26" s="38"/>
-    </row>
-    <row r="27" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M26" s="38"/>
+    </row>
+    <row r="27" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="50">
         <f>ROW(B27) - ROW($B$9)</f>
@@ -2568,19 +2287,9 @@
         <f>K27*5</f>
         <v>20</v>
       </c>
-      <c r="M27" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N27" s="63">
-        <v>0.1</v>
-      </c>
-      <c r="O27" s="62">
-        <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="P27" s="36"/>
-    </row>
-    <row r="28" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M27" s="36"/>
+    </row>
+    <row r="28" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="50">
         <f t="shared" si="0"/>
@@ -2614,22 +2323,12 @@
         <v>1</v>
       </c>
       <c r="L28" s="39">
-        <f t="shared" ref="L28" si="10">K28*5</f>
+        <f t="shared" ref="L28" si="9">K28*5</f>
         <v>5</v>
       </c>
-      <c r="M28" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N28" s="63">
-        <v>0.1</v>
-      </c>
-      <c r="O28" s="62">
-        <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="P28" s="38"/>
-    </row>
-    <row r="29" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M28" s="38"/>
+    </row>
+    <row r="29" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="50">
         <f>ROW(B29) - ROW($B$9)</f>
@@ -2666,19 +2365,9 @@
         <f>K29*5</f>
         <v>20</v>
       </c>
-      <c r="M29" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N29" s="63">
-        <v>0.1</v>
-      </c>
-      <c r="O29" s="62">
-        <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="P29" s="36"/>
-    </row>
-    <row r="30" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M29" s="36"/>
+    </row>
+    <row r="30" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="50">
         <f t="shared" si="0"/>
@@ -2712,22 +2401,12 @@
         <v>2</v>
       </c>
       <c r="L30" s="39">
-        <f t="shared" ref="L30" si="11">K30*5</f>
+        <f t="shared" ref="L30" si="10">K30*5</f>
         <v>10</v>
       </c>
-      <c r="M30" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N30" s="63">
-        <v>0.1</v>
-      </c>
-      <c r="O30" s="62">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="P30" s="38"/>
-    </row>
-    <row r="31" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M30" s="38"/>
+    </row>
+    <row r="31" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="50">
         <f>ROW(B31) - ROW($B$9)</f>
@@ -2764,19 +2443,9 @@
         <f>K31*5</f>
         <v>5</v>
       </c>
-      <c r="M31" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N31" s="63">
-        <v>0.1</v>
-      </c>
-      <c r="O31" s="62">
-        <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="P31" s="36"/>
-    </row>
-    <row r="32" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M31" s="36"/>
+    </row>
+    <row r="32" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="50">
         <f t="shared" si="0"/>
@@ -2810,22 +2479,12 @@
         <v>1</v>
       </c>
       <c r="L32" s="39">
-        <f t="shared" ref="L32:L33" si="12">K32*5</f>
+        <f t="shared" ref="L32:L33" si="11">K32*5</f>
         <v>5</v>
       </c>
-      <c r="M32" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N32" s="63">
-        <v>0.1</v>
-      </c>
-      <c r="O32" s="62">
-        <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="P32" s="38"/>
-    </row>
-    <row r="33" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M32" s="38"/>
+    </row>
+    <row r="33" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="50">
         <f t="shared" si="0"/>
@@ -2835,16 +2494,16 @@
         <v>11</v>
       </c>
       <c r="D33" s="36" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="E33" s="36" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="F33" s="36" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="G33" s="36" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="H33" s="36" t="s">
         <v>121</v>
@@ -2853,28 +2512,18 @@
         <v>91</v>
       </c>
       <c r="J33" s="36" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="K33" s="36">
         <v>1</v>
       </c>
       <c r="L33" s="39">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="M33" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N33" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="O33" s="62">
-        <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="P33" s="36"/>
-    </row>
-    <row r="34" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M33" s="36"/>
+    </row>
+    <row r="34" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="50">
         <f>ROW(B34) - ROW($B$9)</f>
@@ -2911,19 +2560,9 @@
         <f>K34*5</f>
         <v>5</v>
       </c>
-      <c r="M34" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N34" s="62">
-        <v>3.85</v>
-      </c>
-      <c r="O34" s="62">
-        <f t="shared" si="2"/>
-        <v>19.25</v>
-      </c>
-      <c r="P34" s="36"/>
-    </row>
-    <row r="35" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M34" s="36"/>
+    </row>
+    <row r="35" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="50">
         <f>ROW(B35) - ROW($B$9)</f>
@@ -2960,42 +2599,34 @@
         <f>K35*5</f>
         <v>5</v>
       </c>
-      <c r="M35" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="N35" s="62">
-        <v>0.59</v>
-      </c>
-      <c r="O35" s="62">
-        <f t="shared" si="2"/>
-        <v>2.9499999999999997</v>
-      </c>
-      <c r="P35" s="36"/>
-    </row>
-    <row r="36" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M35" s="36"/>
+    </row>
+    <row r="36" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="50">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
       <c r="C36" s="57" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="D36" s="36" t="s">
         <v>121</v>
       </c>
       <c r="E36" s="36" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="F36" s="36" t="s">
         <v>121</v>
       </c>
       <c r="G36" s="36" t="s">
-        <v>153</v>
-      </c>
-      <c r="H36" s="70"/>
+        <v>145</v>
+      </c>
+      <c r="H36" s="61" t="s">
+        <v>121</v>
+      </c>
       <c r="I36" s="36" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="J36" s="36" t="s">
         <v>121</v>
@@ -3003,21 +2634,12 @@
       <c r="K36" s="36">
         <v>1</v>
       </c>
-      <c r="L36" s="70">
+      <c r="L36" s="61">
         <v>5</v>
       </c>
-      <c r="M36" s="61" t="s">
-        <v>132</v>
-      </c>
-      <c r="N36" s="63" t="s">
-        <v>121</v>
-      </c>
-      <c r="O36" s="62" t="s">
-        <v>121</v>
-      </c>
-      <c r="P36" s="71"/>
-    </row>
-    <row r="37" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M36" s="36"/>
+    </row>
+    <row r="37" spans="1:13" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="31"/>
       <c r="C37" s="48"/>
@@ -3029,18 +2651,10 @@
       <c r="I37" s="34"/>
       <c r="J37" s="35"/>
       <c r="K37" s="35"/>
-      <c r="L37" s="75" t="s">
-        <v>133</v>
-      </c>
-      <c r="M37" s="76"/>
-      <c r="N37" s="76"/>
-      <c r="O37" s="65">
-        <f>SUM(O10:O35)</f>
-        <v>88.4</v>
-      </c>
-      <c r="P37" s="41"/>
-    </row>
-    <row r="38" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L37" s="62"/>
+      <c r="M37" s="41"/>
+    </row>
+    <row r="38" spans="1:13" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="24"/>
       <c r="C38" s="49"/>
@@ -3052,51 +2666,16 @@
       <c r="I38" s="9"/>
       <c r="J38" s="9"/>
       <c r="K38" s="9"/>
-      <c r="L38" s="75" t="s">
-        <v>134</v>
-      </c>
-      <c r="M38" s="76"/>
-      <c r="N38" s="76"/>
-      <c r="O38" s="66">
-        <f>O37/5</f>
-        <v>17.68</v>
-      </c>
-      <c r="P38" s="42"/>
+      <c r="L38" s="62"/>
+      <c r="M38" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="J1:P1"/>
-    <mergeCell ref="P3:P8"/>
-    <mergeCell ref="L37:N37"/>
-    <mergeCell ref="L38:N38"/>
+  <mergeCells count="2">
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="M3:M8"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="M10" r:id="rId1"/>
-    <hyperlink ref="M11" r:id="rId2"/>
-    <hyperlink ref="M12" r:id="rId3"/>
-    <hyperlink ref="M14" r:id="rId4"/>
-    <hyperlink ref="M15" r:id="rId5"/>
-    <hyperlink ref="M16" r:id="rId6"/>
-    <hyperlink ref="M17" r:id="rId7"/>
-    <hyperlink ref="M19" r:id="rId8"/>
-    <hyperlink ref="M23" r:id="rId9"/>
-    <hyperlink ref="M24" r:id="rId10"/>
-    <hyperlink ref="M26" r:id="rId11"/>
-    <hyperlink ref="M27" r:id="rId12"/>
-    <hyperlink ref="M28" r:id="rId13"/>
-    <hyperlink ref="M29" r:id="rId14"/>
-    <hyperlink ref="M30" r:id="rId15"/>
-    <hyperlink ref="M31" r:id="rId16"/>
-    <hyperlink ref="M32" r:id="rId17"/>
-    <hyperlink ref="M34" r:id="rId18"/>
-    <hyperlink ref="M35" r:id="rId19"/>
-    <hyperlink ref="M20" r:id="rId20"/>
-    <hyperlink ref="M25" r:id="rId21"/>
-    <hyperlink ref="M33" r:id="rId22"/>
-    <hyperlink ref="M18" r:id="rId23"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId24"/>
-  <drawing r:id="rId25"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>